<commit_message>
Updated the OpenAi for check the performace issues
</commit_message>
<xml_diff>
--- a/python/table_metadata.xlsx
+++ b/python/table_metadata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="10440" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="9840" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="317">
   <si>
     <t>TableName</t>
   </si>
@@ -53,223 +53,222 @@
     <t>Core work order records. Central table — almost every query involves this table. Each WO belongs to a project and an office.</t>
   </si>
   <si>
+    <t>WorkOrderNumber</t>
+  </si>
+  <si>
+    <t>Id is INTEGER PK for JOINs. WorkOrderNumber is TEXT never use as integer. IsDeleted=false for active. OfficeId is NULL for all records — NEVER USE OfficeId. branches = AbpOrganizationUnits table. organizations = AbpOrganizationUnits table. For location/branch/office/fort myers queries always JOIN AbpOrganizationUnits ON OrganizationId=Id and filter by DisplayName ILIKE. For count by group always use COUNT(Id) with GROUP BY. For project-wise counts use ProjectId -&gt; Projects. For phase-wise counts use PhaseId -&gt; Phases. For day-wise/daily count queries use: COUNT("WorkOrders"."Id") GROUP BY "WorkOrders"."CreationTime"::date ORDER BY date. For per-day results always cast timestamp to date using ::date. Always SELECT WorkOrderNumber and Subject for display.</t>
+  </si>
+  <si>
+    <t>Offices</t>
+  </si>
+  <si>
+    <t>Office/branch locations. Work orders and projects are linked to an office via OfficeId.</t>
+  </si>
+  <si>
+    <t>OfficeName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEVER JOIN this table for location filtering. OfficeId is NULL in WorkOrders and Projects. For any location/branch/city/office name filter always use AbpOrganizationUnits table instead.Offices are also called BRANCHES. Use OfficeName for display and filtering with ILIKE. To count WOs by branch: JOIN WorkOrders ON OfficeId=Id, GROUP BY OfficeName. IsDeleted=false. </t>
+  </si>
+  <si>
+    <t>AbpUsers</t>
+  </si>
+  <si>
+    <t>All users in the system: field users, project managers, admins, technicians.</t>
+  </si>
+  <si>
+    <t>UserName</t>
+  </si>
+  <si>
+    <t>IsActive=true for active users. Use UserName for filtering by login. Name+Surname for full name. To get users by role JOIN AbpUserRoles then AbpRoles.</t>
+  </si>
+  <si>
+    <t>AbpRoles</t>
+  </si>
+  <si>
+    <t>Role definitions. Name column contains GUIDs — NEVER use Name for filtering or display.</t>
+  </si>
+  <si>
+    <t>DisplayName</t>
+  </si>
+  <si>
+    <t>CRITICAL: ALWAYS use DisplayName for both SELECT and WHERE. Name column is GUID not readable. Known roles: Admin, User, Field User, Project Manager, Engineer of Record, Lab Manager, Dispatcher</t>
+  </si>
+  <si>
+    <t>AbpUserRoles</t>
+  </si>
+  <si>
+    <t>Junction table mapping users to roles. Use to find which users have a specific role.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>NO IsDeleted column — filter active users via AbpUsers.IsActive=true. JOIN AbpUsers ON UserId=AbpUsers.Id and JOIN AbpRoles ON RoleId=AbpRoles.Id</t>
+  </si>
+  <si>
+    <t>WorkOrderTests</t>
+  </si>
+  <si>
+    <t>Individual tests performed within a work order. One WO can have many tests.</t>
+  </si>
+  <si>
+    <t>WorkOrderId is INTEGER FK to WorkOrders.Id — not WorkOrderNumber. RecordId links to SampleSpecimens.Id for specimen data.</t>
+  </si>
+  <si>
+    <t>WorkOrderUsers</t>
+  </si>
+  <si>
+    <t>Users explicitly assigned to a work order. Tracks acceptance and rejection.</t>
+  </si>
+  <si>
+    <t>NO IsDeleted column. Filter via WorkOrders.IsDeleted. UserId-&gt;AbpUsers.Id, WorkOrderId-&gt;WorkOrders.Id</t>
+  </si>
+  <si>
+    <t>WorkOrderEquipments</t>
+  </si>
+  <si>
+    <t>Equipment items assigned to a work order.</t>
+  </si>
+  <si>
+    <t>WorkOrderId-&gt;WorkOrders.Id, EquipmentId-&gt;Equipments.Id</t>
+  </si>
+  <si>
+    <t>SampleSpecimens</t>
+  </si>
+  <si>
+    <t>Physical specimens for lab testing. NOTE: The Specimens table is EMPTY — always use SampleSpecimens.</t>
+  </si>
+  <si>
+    <t>SpecimenNumber</t>
+  </si>
+  <si>
+    <t>Does NOT link directly to WorkOrders. Path: WorkOrders -&gt; WorkOrderTests.RecordId -&gt; SampleSpecimens.Id. SampleId-&gt;Samples.Id, ProjectId-&gt;Projects.Id</t>
+  </si>
+  <si>
+    <t>FormWorkFlowStates</t>
+  </si>
+  <si>
+    <t>Tracks workflow state history of forms within work orders.</t>
+  </si>
+  <si>
+    <t>WorkOrderId-&gt;WorkOrders.Id, FormId-&gt;Forms.Id, UserId-&gt;AbpUsers.Id (user who changed state)</t>
+  </si>
+  <si>
+    <t>Clients</t>
+  </si>
+  <si>
+    <t>Client companies that own projects.</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>IsDeleted=false for active. ClientId in Projects and WorkOrders links here.</t>
+  </si>
+  <si>
+    <t>Equipments</t>
+  </si>
+  <si>
+    <t>Equipment items used in field work orders.</t>
+  </si>
+  <si>
+    <t>Referenced by WorkOrderEquipments.EquipmentId</t>
+  </si>
+  <si>
+    <t>Forms</t>
+  </si>
+  <si>
+    <t>Test form templates used in work orders.</t>
+  </si>
+  <si>
+    <t>Referenced by WorkOrderTests.FormId and FormWorkFlowStates.FormId</t>
+  </si>
+  <si>
+    <t>Phases</t>
+  </si>
+  <si>
+    <t>Project phases. WorkOrders.PhaseId links here.</t>
+  </si>
+  <si>
+    <t>PhaseName</t>
+  </si>
+  <si>
+    <t>Use PhaseName for display and GROUP BY. PhaseId in WorkOrders links here.</t>
+  </si>
+  <si>
+    <t>Regions</t>
+  </si>
+  <si>
+    <t>Geographic regions.</t>
+  </si>
+  <si>
+    <t>Departments</t>
+  </si>
+  <si>
+    <t>Departments within the organization.</t>
+  </si>
+  <si>
+    <t>IsDeleted=false for active</t>
+  </si>
+  <si>
+    <t>AbpOrganizationUnits</t>
+  </si>
+  <si>
+    <t>Organization hierarchy units: regions, divisions. WorkOrders.OrganizationId and Projects.OrganizationId link here. Organization hierarchy units. WorkOrders.OrganizationId links here. Represents branches and organizations.</t>
+  </si>
+  <si>
+    <t>THIS is the correct table for ALL location queries. Use DisplayName ILIKE for filtering by office name, city, branch or any location. JOIN via WorkOrders.OrganizationId or Projects.OrganizationId. Any office name like Charleston, Fort Myers etc will be in DisplayName column of this table. Organizations are also called ORG UNITS. Use DisplayName for display and ILIKE filtering. To count WOs by organization: JOIN WorkOrders ON OrganizationId=Id, GROUP BY DisplayName.Use DisplayName for display and ILIKE filtering. To count WOs by org: JOIN WorkOrders ON OrganizationId=Id GROUP BY DisplayName. branches and organizations both use this table.</t>
+  </si>
+  <si>
+    <t>AbpOrganizationUnitRoles</t>
+  </si>
+  <si>
+    <t>Maps roles to organization units.</t>
+  </si>
+  <si>
+    <t>RoleId-&gt;AbpRoles.Id, OrganizationUnitId-&gt;AbpOrganizationUnits.Id</t>
+  </si>
+  <si>
+    <t>AbpPermissions</t>
+  </si>
+  <si>
+    <t>Permission grants for roles and users.</t>
+  </si>
+  <si>
+    <t>RoleId-&gt;AbpRoles.Id, UserId-&gt;AbpUsers.Id. IsGranted=true for active permissions.</t>
+  </si>
+  <si>
+    <t>Projects</t>
+  </si>
+  <si>
+    <t>Stores all projects. Each project belongs to a client, office and organization. Work orders link to projects via ProjectId. Stores all projects. Each project belongs to a client, office and has an assigned Project Manager.</t>
+  </si>
+  <si>
+    <t>ProjectName</t>
+  </si>
+  <si>
+    <t>OfficeId is NULL for all records — NEVER USE OfficeId. For location/office/branch queries always JOIN AbpOrganizationUnits ON Projects.OrganizationId=AbpOrganizationUnits.Id and filter by DisplayName ILIKE.Use ProjectName for display. ProjectNumber is human-readable lookup. IsDeleted=false for active. PMUserId links to Project Manager in AbpUsers. CreatorUserId links to AbpUsers. For project-wise WO count: JOIN WorkOrders ON ProjectId=Projects.Id GROUP BY ProjectName. Use ProjectName for display. ProjectNumber is human-readable lookup ID. IsDeleted=false for active. PMUserId links to AbpUsers.Id. For project-wise WO count: JOIN WorkOrders ON WorkOrders.ProjectId=Projects.Id GROUP BY ProjectName. CreatorUserId and PMUserId are INTEGER FKs — NEVER filter by username directly, always JOIN AbpUsers.</t>
+  </si>
+  <si>
+    <t>ColumnName</t>
+  </si>
+  <si>
+    <t>Relationship</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>Primary key INTEGER. Use in all JOINs. NOT same as WorkOrderNumber.</t>
+  </si>
+  <si>
     <t>Subject</t>
   </si>
   <si>
-    <t xml:space="preserve">Id is INTEGER PK for JOINs. WorkOrderNumber is TEXT never use as integer. IsDeleted=false for active. branches = Offices table. organizations = AbpOrganizationUnits table. For count by group always use COUNT(Id) with GROUP BY. For project-wise counts use ProjectId -&gt; Projects. For phase-wise counts use PhaseId -&gt; Phases. For day-wise/daily count queries use: COUNT("WorkOrders"."Id") GROUP BY "WorkOrders"."CreationTime"::date ORDER BY date. For per-day results always cast timestamp to date using ::date.
-</t>
-  </si>
-  <si>
-    <t>Offices</t>
-  </si>
-  <si>
-    <t>Office/branch locations. Work orders and projects are linked to an office via OfficeId.</t>
-  </si>
-  <si>
-    <t>OfficeName</t>
-  </si>
-  <si>
-    <t>Offices are also called BRANCHES. Use OfficeName for display and filtering with ILIKE. To count WOs by branch: JOIN WorkOrders ON OfficeId=Id, GROUP BY OfficeName. IsDeleted=false.</t>
-  </si>
-  <si>
-    <t>AbpUsers</t>
-  </si>
-  <si>
-    <t>All users in the system: field users, project managers, admins, technicians.</t>
-  </si>
-  <si>
-    <t>UserName</t>
-  </si>
-  <si>
-    <t>IsActive=true for active users. Use UserName for filtering by login. Name+Surname for full name. To get users by role JOIN AbpUserRoles then AbpRoles.</t>
-  </si>
-  <si>
-    <t>AbpRoles</t>
-  </si>
-  <si>
-    <t>Role definitions. Name column contains GUIDs — NEVER use Name for filtering or display.</t>
-  </si>
-  <si>
-    <t>DisplayName</t>
-  </si>
-  <si>
-    <t>CRITICAL: ALWAYS use DisplayName for both SELECT and WHERE. Name column is GUID not readable. Known roles: Admin, User, Field User, Project Manager, Engineer of Record, Lab Manager, Dispatcher</t>
-  </si>
-  <si>
-    <t>AbpUserRoles</t>
-  </si>
-  <si>
-    <t>Junction table mapping users to roles. Use to find which users have a specific role.</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>NO IsDeleted column — filter active users via AbpUsers.IsActive=true. JOIN AbpUsers ON UserId=AbpUsers.Id and JOIN AbpRoles ON RoleId=AbpRoles.Id</t>
-  </si>
-  <si>
-    <t>WorkOrderTests</t>
-  </si>
-  <si>
-    <t>Individual tests performed within a work order. One WO can have many tests.</t>
-  </si>
-  <si>
-    <t>WorkOrderId is INTEGER FK to WorkOrders.Id — not WorkOrderNumber. RecordId links to SampleSpecimens.Id for specimen data.</t>
-  </si>
-  <si>
-    <t>WorkOrderUsers</t>
-  </si>
-  <si>
-    <t>Users explicitly assigned to a work order. Tracks acceptance and rejection.</t>
-  </si>
-  <si>
-    <t>NO IsDeleted column. Filter via WorkOrders.IsDeleted. UserId-&gt;AbpUsers.Id, WorkOrderId-&gt;WorkOrders.Id</t>
-  </si>
-  <si>
-    <t>WorkOrderEquipments</t>
-  </si>
-  <si>
-    <t>Equipment items assigned to a work order.</t>
-  </si>
-  <si>
-    <t>WorkOrderId-&gt;WorkOrders.Id, EquipmentId-&gt;Equipments.Id</t>
-  </si>
-  <si>
-    <t>SampleSpecimens</t>
-  </si>
-  <si>
-    <t>Physical specimens for lab testing. NOTE: The Specimens table is EMPTY — always use SampleSpecimens.</t>
-  </si>
-  <si>
-    <t>SpecimenNumber</t>
-  </si>
-  <si>
-    <t>Does NOT link directly to WorkOrders. Path: WorkOrders -&gt; WorkOrderTests.RecordId -&gt; SampleSpecimens.Id. SampleId-&gt;Samples.Id, ProjectId-&gt;Projects.Id</t>
-  </si>
-  <si>
-    <t>FormWorkFlowStates</t>
-  </si>
-  <si>
-    <t>Tracks workflow state history of forms within work orders.</t>
-  </si>
-  <si>
-    <t>WorkOrderId-&gt;WorkOrders.Id, FormId-&gt;Forms.Id, UserId-&gt;AbpUsers.Id (user who changed state)</t>
-  </si>
-  <si>
-    <t>Clients</t>
-  </si>
-  <si>
-    <t>Client companies that own projects.</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>IsDeleted=false for active. ClientId in Projects and WorkOrders links here.</t>
-  </si>
-  <si>
-    <t>Equipments</t>
-  </si>
-  <si>
-    <t>Equipment items used in field work orders.</t>
-  </si>
-  <si>
-    <t>Referenced by WorkOrderEquipments.EquipmentId</t>
-  </si>
-  <si>
-    <t>Forms</t>
-  </si>
-  <si>
-    <t>Test form templates used in work orders.</t>
-  </si>
-  <si>
-    <t>Referenced by WorkOrderTests.FormId and FormWorkFlowStates.FormId</t>
-  </si>
-  <si>
-    <t>Phases</t>
-  </si>
-  <si>
-    <t>Project phases. WorkOrders.PhaseId links here.</t>
-  </si>
-  <si>
-    <t>PhaseName</t>
-  </si>
-  <si>
-    <t>Use PhaseName for display and GROUP BY. PhaseId in WorkOrders links here.</t>
-  </si>
-  <si>
-    <t>Regions</t>
-  </si>
-  <si>
-    <t>Geographic regions.</t>
-  </si>
-  <si>
-    <t>Departments</t>
-  </si>
-  <si>
-    <t>Departments within the organization.</t>
-  </si>
-  <si>
-    <t>IsDeleted=false for active</t>
-  </si>
-  <si>
-    <t>AbpOrganizationUnits</t>
-  </si>
-  <si>
-    <t>Organization hierarchy units: regions, divisions. WorkOrders.OrganizationId and Projects.OrganizationId link here. Organization hierarchy units. WorkOrders.OrganizationId links here. Represents branches and organizations.</t>
-  </si>
-  <si>
-    <t>Organizations are also called ORG UNITS. Use DisplayName for display and ILIKE filtering. To count WOs by organization: JOIN WorkOrders ON OrganizationId=Id, GROUP BY DisplayName.Use DisplayName for display and ILIKE filtering. To count WOs by org: JOIN WorkOrders ON OrganizationId=Id GROUP BY DisplayName. branches and organizations both use this table.</t>
-  </si>
-  <si>
-    <t>AbpOrganizationUnitRoles</t>
-  </si>
-  <si>
-    <t>Maps roles to organization units.</t>
-  </si>
-  <si>
-    <t>RoleId-&gt;AbpRoles.Id, OrganizationUnitId-&gt;AbpOrganizationUnits.Id</t>
-  </si>
-  <si>
-    <t>AbpPermissions</t>
-  </si>
-  <si>
-    <t>Permission grants for roles and users.</t>
-  </si>
-  <si>
-    <t>RoleId-&gt;AbpRoles.Id, UserId-&gt;AbpUsers.Id. IsGranted=true for active permissions.</t>
-  </si>
-  <si>
-    <t>Projects</t>
-  </si>
-  <si>
-    <t>Stores all projects. Each project belongs to a client, office and organization. Work orders link to projects via ProjectId. Stores all projects. Each project belongs to a client, office and has an assigned Project Manager.</t>
-  </si>
-  <si>
-    <t>ProjectName</t>
-  </si>
-  <si>
-    <t>Use ProjectName for display. ProjectNumber is human-readable lookup. IsDeleted=false for active. PMUserId links to Project Manager in AbpUsers. CreatorUserId links to AbpUsers. For project-wise WO count: JOIN WorkOrders ON ProjectId=Projects.Id GROUP BY ProjectName. Use ProjectName for display. ProjectNumber is human-readable lookup ID. IsDeleted=false for active. PMUserId links to AbpUsers.Id. For project-wise WO count: JOIN WorkOrders ON WorkOrders.ProjectId=Projects.Id GROUP BY ProjectName. CreatorUserId and PMUserId are INTEGER FKs — NEVER filter by username directly, always JOIN AbpUsers.</t>
-  </si>
-  <si>
-    <t>ColumnName</t>
-  </si>
-  <si>
-    <t>Relationship</t>
-  </si>
-  <si>
-    <t>Id</t>
-  </si>
-  <si>
-    <t>Primary key INTEGER. Use in all JOINs. NOT same as WorkOrderNumber.</t>
-  </si>
-  <si>
     <t>Work order title/name. ALWAYS USE FOR DISPLAY.</t>
   </si>
   <si>
-    <t>WorkOrderNumber</t>
-  </si>
-  <si>
     <t>Human-readable TEXT ID e.g. 08.25001260. Use only for WHERE lookups by number — never as integer FK.</t>
   </si>
   <si>
@@ -291,7 +290,7 @@
     <t>OfficeId</t>
   </si>
   <si>
-    <t>NULL for all records — NEVER USE. Use OrganizationId for all location queries.</t>
+    <t>OfficeId is NULL for all records — NEVER USE OfficeId. Use OrganizationId -&gt; AbpOrganizationUnits for all location/office/branch queries.</t>
   </si>
   <si>
     <t>ClientId</t>
@@ -399,7 +398,7 @@
     <t>Linked client.</t>
   </si>
   <si>
-    <t>Linked office.</t>
+    <t>NULL for all records — NEVER USE. Use OrganizationId -&gt; AbpOrganizationUnits for all location queries.</t>
   </si>
   <si>
     <t>-&gt; Offices.Id</t>
@@ -930,7 +929,7 @@
     <t>project,projects</t>
   </si>
   <si>
-    <t>office,offices,branch,branches,fort,myers,charleston,location</t>
+    <t>organization,organizations,org,unit,units,branch,branches,location</t>
   </si>
   <si>
     <t>user,users,username,creator,created,technician,active</t>
@@ -940,9 +939,6 @@
   </si>
   <si>
     <t>phase,phases</t>
-  </si>
-  <si>
-    <t>organization,organizations,org,unit,units,branch,branches,location</t>
   </si>
   <si>
     <t>specimen,sample,test,tests</t>
@@ -1633,7 +1629,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1650,6 +1646,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="distributed" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="distributed"/>
@@ -2014,26 +2013,26 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="65" style="8" customWidth="1"/>
+    <col min="2" max="2" width="65" style="9" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="70" style="8" customWidth="1"/>
+    <col min="4" max="4" width="70" style="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1" spans="1:4">
+    <row r="2" s="10" customFormat="1" ht="144" customHeight="1" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -2047,7 +2046,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1" spans="1:4">
+    <row r="3" ht="64" customHeight="1" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -2225,7 +2224,7 @@
       <c r="C15" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="9" t="s">
         <v>53</v>
       </c>
     </row>
@@ -2275,10 +2274,10 @@
       <c r="A19" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="9" t="s">
         <v>64</v>
       </c>
     </row>
@@ -2286,27 +2285,27 @@
       <c r="A20" t="s">
         <v>65</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="9" t="s">
         <v>66</v>
       </c>
       <c r="C20" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="9" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="21" ht="129.6" spans="1:4">
+    <row r="21" ht="158.4" spans="1:4">
       <c r="A21" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="9" t="s">
         <v>69</v>
       </c>
       <c r="C21" t="s">
         <v>70</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="9" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2342,271 +2341,271 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1" spans="1:4">
+    <row r="2" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="2" t="s">
         <v>75</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1" spans="1:4">
+    <row r="3" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="6" t="s">
         <v>76</v>
       </c>
+      <c r="C3" s="3" t="s">
+        <v>77</v>
+      </c>
       <c r="D3" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1" spans="1:4">
+    <row r="4" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" spans="1:4">
+    <row r="5" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="3" t="s">
         <v>80</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" spans="1:4">
+    <row r="6" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="2" t="s">
         <v>82</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" spans="1:4">
+    <row r="7" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="3" t="s">
         <v>85</v>
       </c>
       <c r="D7" s="3"/>
     </row>
-    <row r="8" ht="30" customHeight="1" spans="1:4">
+    <row r="8" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="2" t="s">
         <v>87</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1" spans="1:4">
+    <row r="9" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1" spans="1:4">
+    <row r="10" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A10" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="3" t="s">
         <v>93</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1" spans="1:4">
+    <row r="11" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A11" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1" spans="1:4">
+    <row r="12" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A12" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="2" t="s">
         <v>97</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1" spans="1:4">
+    <row r="13" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A13" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="3" t="s">
         <v>100</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1" spans="1:4">
+    <row r="14" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="3" t="s">
         <v>103</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" spans="1:4">
+    <row r="15" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A15" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="2" t="s">
         <v>105</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1" spans="1:4">
+    <row r="16" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A16" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="2" t="s">
         <v>107</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1" spans="1:4">
+    <row r="17" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A17" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="3" t="s">
         <v>109</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1" spans="1:4">
+    <row r="18" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A18" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="3" t="s">
         <v>111</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1" spans="1:4">
+    <row r="19" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A19" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="2" t="s">
         <v>113</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1" spans="1:4">
+    <row r="20" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A20" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="3" t="s">
         <v>115</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="21" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="21" ht="30" customHeight="1" spans="1:4">
       <c r="A21" s="2" t="s">
         <v>68</v>
       </c>
@@ -2620,7 +2619,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="22" ht="30" customHeight="1" spans="1:4">
       <c r="A22" s="3" t="s">
         <v>68</v>
       </c>
@@ -2634,7 +2633,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="23" ht="30" customHeight="1" spans="1:4">
       <c r="A23" s="2" t="s">
         <v>68</v>
       </c>
@@ -2648,7 +2647,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="24" ht="30" customHeight="1" spans="1:4">
       <c r="A24" s="3" t="s">
         <v>68</v>
       </c>
@@ -2662,7 +2661,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="25" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="25" ht="30" customHeight="1" spans="1:4">
       <c r="A25" s="2" t="s">
         <v>68</v>
       </c>
@@ -2676,7 +2675,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="26" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="26" ht="30" customHeight="1" spans="1:4">
       <c r="A26" s="3" t="s">
         <v>68</v>
       </c>
@@ -2690,7 +2689,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="27" ht="30" customHeight="1" spans="1:4">
       <c r="A27" s="2" t="s">
         <v>68</v>
       </c>
@@ -2704,7 +2703,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="28" ht="30" customHeight="1" spans="1:4">
       <c r="A28" s="3" t="s">
         <v>68</v>
       </c>
@@ -2718,7 +2717,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="29" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="29" ht="30" customHeight="1" spans="1:4">
       <c r="A29" s="2" t="s">
         <v>68</v>
       </c>
@@ -2732,7 +2731,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="30" ht="30" customHeight="1" spans="1:4">
       <c r="A30" s="3" t="s">
         <v>68</v>
       </c>
@@ -3306,7 +3305,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="71" ht="30" customHeight="1" spans="1:4">
+    <row r="71" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A71" t="s">
         <v>4</v>
       </c>
@@ -3316,7 +3315,7 @@
       <c r="C71" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="D71" s="11" t="s">
+      <c r="D71" s="12" t="s">
         <v>125</v>
       </c>
     </row>
@@ -3327,7 +3326,7 @@
       <c r="B72" t="s">
         <v>18</v>
       </c>
-      <c r="C72" s="7" t="s">
+      <c r="C72" s="8" t="s">
         <v>197</v>
       </c>
     </row>
@@ -3342,14 +3341,14 @@
         <v>198</v>
       </c>
     </row>
-    <row r="74" spans="1:4">
+    <row r="74" hidden="1" spans="1:4">
       <c r="A74" t="s">
         <v>4</v>
       </c>
       <c r="B74" t="s">
         <v>199</v>
       </c>
-      <c r="C74" s="4" t="s">
+      <c r="C74" s="9" t="s">
         <v>200</v>
       </c>
       <c r="D74" t="s">
@@ -3367,14 +3366,14 @@
         <v>202</v>
       </c>
     </row>
-    <row r="76" ht="28.8" hidden="1" spans="1:4">
+    <row r="76" hidden="1" spans="1:4">
       <c r="A76" t="s">
         <v>50</v>
       </c>
       <c r="B76" t="s">
         <v>52</v>
       </c>
-      <c r="C76" s="8" t="s">
+      <c r="C76" s="9" t="s">
         <v>203</v>
       </c>
     </row>
@@ -3400,14 +3399,14 @@
         <v>205</v>
       </c>
     </row>
-    <row r="79" ht="28.8" hidden="1" spans="1:4">
+    <row r="79" hidden="1" spans="1:4">
       <c r="A79" t="s">
         <v>59</v>
       </c>
       <c r="B79" t="s">
         <v>18</v>
       </c>
-      <c r="C79" s="8" t="s">
+      <c r="C79" s="9" t="s">
         <v>206</v>
       </c>
     </row>
@@ -3547,29 +3546,29 @@
         <v>91</v>
       </c>
     </row>
-    <row r="91" ht="115.2" spans="1:4">
+    <row r="91" ht="72" hidden="1" spans="1:4">
       <c r="A91" t="s">
         <v>4</v>
       </c>
       <c r="B91" t="s">
         <v>219</v>
       </c>
-      <c r="C91" s="8" t="s">
+      <c r="C91" s="9" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="92" spans="1:4">
+    <row r="92" hidden="1" spans="1:4">
       <c r="A92" t="s">
         <v>4</v>
       </c>
       <c r="B92" t="s">
         <v>221</v>
       </c>
-      <c r="C92" s="4" t="s">
+      <c r="C92" s="9" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="93" hidden="1" spans="1:4">
+    <row r="93" spans="1:4">
       <c r="A93" t="s">
         <v>68</v>
       </c>
@@ -3580,7 +3579,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="94" hidden="1" spans="1:4">
+    <row r="94" spans="1:4">
       <c r="A94" t="s">
         <v>68</v>
       </c>
@@ -3591,7 +3590,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="95" hidden="1" spans="1:4">
+    <row r="95" spans="1:4">
       <c r="A95" t="s">
         <v>68</v>
       </c>
@@ -3602,7 +3601,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="96" hidden="1" spans="1:4">
+    <row r="96" spans="1:4">
       <c r="A96" t="s">
         <v>68</v>
       </c>
@@ -3613,7 +3612,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="97" hidden="1" spans="1:4">
+    <row r="97" spans="1:4">
       <c r="A97" t="s">
         <v>68</v>
       </c>
@@ -3624,7 +3623,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="98" hidden="1" spans="1:4">
+    <row r="98" spans="1:4">
       <c r="A98" t="s">
         <v>68</v>
       </c>
@@ -3635,7 +3634,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="99" hidden="1" spans="1:4">
+    <row r="99" spans="1:4">
       <c r="A99" t="s">
         <v>68</v>
       </c>
@@ -3649,35 +3648,35 @@
         <v>83</v>
       </c>
     </row>
-    <row r="100" ht="28.8" hidden="1" spans="1:4">
+    <row r="100" ht="28.8" spans="1:4">
       <c r="A100" t="s">
         <v>68</v>
       </c>
       <c r="B100" t="s">
         <v>126</v>
       </c>
-      <c r="C100" s="8" t="s">
+      <c r="C100" s="9" t="s">
         <v>236</v>
       </c>
       <c r="D100" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="101" ht="28.8" hidden="1" spans="1:4">
+    <row r="101" ht="28.8" spans="1:4">
       <c r="A101" t="s">
         <v>68</v>
       </c>
       <c r="B101" t="s">
         <v>89</v>
       </c>
-      <c r="C101" s="8" t="s">
+      <c r="C101" s="9" t="s">
         <v>237</v>
       </c>
       <c r="D101" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="102" ht="28.8" hidden="1" spans="1:4">
+    <row r="102" spans="1:4">
       <c r="A102" t="s">
         <v>68</v>
       </c>
@@ -3688,7 +3687,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="103" ht="28.8" spans="1:4">
+    <row r="103" hidden="1" spans="1:4">
       <c r="A103" t="s">
         <v>4</v>
       </c>
@@ -3699,7 +3698,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="104" ht="28.8" hidden="1" spans="1:4">
+    <row r="104" hidden="1" spans="1:4">
       <c r="A104" t="s">
         <v>12</v>
       </c>
@@ -3710,7 +3709,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="105" ht="28.8" hidden="1" spans="1:4">
+    <row r="105" hidden="1" spans="1:4">
       <c r="A105" t="s">
         <v>59</v>
       </c>
@@ -3721,7 +3720,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="106" ht="28.8" hidden="1" spans="1:4">
+    <row r="106" hidden="1" spans="1:4">
       <c r="A106" t="s">
         <v>8</v>
       </c>
@@ -3732,7 +3731,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="107" ht="28.8" hidden="1" spans="1:4">
+    <row r="107" hidden="1" spans="1:4">
       <c r="A107" t="s">
         <v>16</v>
       </c>
@@ -3754,7 +3753,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="109" ht="28.8" hidden="1" spans="1:4">
+    <row r="109" hidden="1" spans="1:4">
       <c r="A109" t="s">
         <v>50</v>
       </c>
@@ -3769,7 +3768,7 @@
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D109" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
       <filters>
-        <filter val="WorkOrders"/>
+        <filter val="Projects"/>
       </filters>
     </filterColumn>
     <extLst/>
@@ -4563,7 +4562,7 @@
         <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="C9" t="s">
         <v>296</v>
@@ -4574,7 +4573,7 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C10" t="s">
         <v>296</v>
@@ -4585,7 +4584,7 @@
         <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C11" t="s">
         <v>296</v>
@@ -4596,7 +4595,7 @@
         <v>47</v>
       </c>
       <c r="B12" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C12" t="s">
         <v>296</v>
@@ -4607,7 +4606,7 @@
         <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C13" t="s">
         <v>296</v>
@@ -4618,7 +4617,7 @@
         <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C14" t="s">
         <v>296</v>
@@ -4629,10 +4628,10 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
+        <v>307</v>
+      </c>
+      <c r="C15" t="s">
         <v>308</v>
-      </c>
-      <c r="C15" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -4640,32 +4639,32 @@
         <v>37</v>
       </c>
       <c r="B16" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C16" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
+        <v>310</v>
+      </c>
+      <c r="B17" t="s">
         <v>311</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>312</v>
-      </c>
-      <c r="C17" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>313</v>
+      </c>
+      <c r="B18" t="s">
         <v>314</v>
       </c>
-      <c r="B18" t="s">
-        <v>315</v>
-      </c>
       <c r="C18" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -4673,10 +4672,10 @@
         <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C19" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -4684,10 +4683,10 @@
         <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C20" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed the voice search
</commit_message>
<xml_diff>
--- a/python/table_metadata.xlsx
+++ b/python/table_metadata.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="316">
   <si>
     <t>TableName</t>
   </si>
@@ -263,10 +263,7 @@
     <t>Primary key INTEGER. Use in all JOINs. NOT same as WorkOrderNumber.</t>
   </si>
   <si>
-    <t>Subject</t>
-  </si>
-  <si>
-    <t>Work order title/name. ALWAYS USE FOR DISPLAY.</t>
+    <t>Primary display column for work orders. ALWAYS USE THIS for listing and display. Human-readable ID e.g. 08.25001260.</t>
   </si>
   <si>
     <t>Human-readable TEXT ID e.g. 08.25001260. Use only for WHERE lookups by number — never as integer FK.</t>
@@ -2341,7 +2338,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="2" ht="30" customHeight="1" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -2355,21 +2352,21 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="3" ht="30" customHeight="1" spans="1:4">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="D3" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="4" ht="30" customHeight="1" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -2377,235 +2374,235 @@
         <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="5" ht="30" customHeight="1" spans="1:4">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="D5" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="6" ht="30" customHeight="1" spans="1:4">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="7" ht="30" hidden="1" customHeight="1" spans="1:4">
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:4">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>85</v>
-      </c>
       <c r="D7" s="3"/>
     </row>
-    <row r="8" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="8" ht="30" customHeight="1" spans="1:4">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" ht="30" hidden="1" customHeight="1" spans="1:4">
+    </row>
+    <row r="9" ht="30" customHeight="1" spans="1:4">
       <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="10" ht="30" hidden="1" customHeight="1" spans="1:4">
+    </row>
+    <row r="10" ht="30" customHeight="1" spans="1:4">
       <c r="A10" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="D10" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="11" ht="30" hidden="1" customHeight="1" spans="1:4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1" spans="1:4">
       <c r="A11" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>95</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" ht="30" hidden="1" customHeight="1" spans="1:4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1" spans="1:4">
       <c r="A12" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="13" ht="30" hidden="1" customHeight="1" spans="1:4">
+    </row>
+    <row r="13" ht="30" customHeight="1" spans="1:4">
       <c r="A13" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="14" ht="30" hidden="1" customHeight="1" spans="1:4">
+    </row>
+    <row r="14" ht="30" customHeight="1" spans="1:4">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>103</v>
-      </c>
       <c r="D14" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="15" ht="30" customHeight="1" spans="1:4">
       <c r="A15" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>105</v>
-      </c>
       <c r="D15" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="16" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="16" ht="30" customHeight="1" spans="1:4">
       <c r="A16" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="D16" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="17" ht="30" customHeight="1" spans="1:4">
       <c r="A17" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>109</v>
-      </c>
       <c r="D17" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="18" ht="30" customHeight="1" spans="1:4">
       <c r="A18" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>111</v>
-      </c>
       <c r="D18" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="19" ht="30" customHeight="1" spans="1:4">
       <c r="A19" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>113</v>
-      </c>
       <c r="D19" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="20" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="20" ht="30" customHeight="1" spans="1:4">
       <c r="A20" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>115</v>
-      </c>
       <c r="D20" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1" spans="1:4">
+    <row r="21" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A21" s="2" t="s">
         <v>68</v>
       </c>
@@ -2613,13 +2610,13 @@
         <v>74</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1" spans="1:4">
+    <row r="22" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A22" s="3" t="s">
         <v>68</v>
       </c>
@@ -2627,119 +2624,119 @@
         <v>70</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1" spans="1:4">
+    <row r="23" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A23" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>119</v>
-      </c>
       <c r="D23" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1" spans="1:4">
+    <row r="24" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A24" s="3" t="s">
         <v>68</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1" spans="1:4">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A25" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C25" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1" spans="1:4">
+    </row>
+    <row r="26" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A26" s="3" t="s">
         <v>68</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="D26" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1" spans="1:4">
+    </row>
+    <row r="27" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A27" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>127</v>
-      </c>
       <c r="D27" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1" spans="1:4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A28" s="3" t="s">
         <v>68</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1" spans="1:4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="29" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A29" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C29" s="5" t="s">
-        <v>130</v>
-      </c>
       <c r="D29" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1" spans="1:4">
+    <row r="30" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A30" s="3" t="s">
         <v>68</v>
       </c>
       <c r="B30" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>132</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>22</v>
@@ -2753,7 +2750,7 @@
         <v>74</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>22</v>
@@ -2767,7 +2764,7 @@
         <v>10</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>22</v>
@@ -2781,7 +2778,7 @@
         <v>18</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>22</v>
@@ -2792,10 +2789,10 @@
         <v>8</v>
       </c>
       <c r="B34" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C34" s="6" t="s">
         <v>136</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>137</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>22</v>
@@ -2806,10 +2803,10 @@
         <v>8</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>138</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>139</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>22</v>
@@ -2820,10 +2817,10 @@
         <v>8</v>
       </c>
       <c r="B36" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>140</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>141</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>22</v>
@@ -2834,10 +2831,10 @@
         <v>8</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>142</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>143</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>22</v>
@@ -2848,10 +2845,10 @@
         <v>8</v>
       </c>
       <c r="B38" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>144</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>145</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>22</v>
@@ -2862,13 +2859,13 @@
         <v>8</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="D39" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="40" ht="30" hidden="1" customHeight="1" spans="1:4">
@@ -2876,10 +2873,10 @@
         <v>8</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>22</v>
@@ -2893,7 +2890,7 @@
         <v>74</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>22</v>
@@ -2907,7 +2904,7 @@
         <v>14</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>22</v>
@@ -2921,7 +2918,7 @@
         <v>42</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>22</v>
@@ -2932,10 +2929,10 @@
         <v>12</v>
       </c>
       <c r="B44" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C44" s="6" t="s">
         <v>153</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>154</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>22</v>
@@ -2946,10 +2943,10 @@
         <v>12</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C45" s="5" t="s">
         <v>155</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>156</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>22</v>
@@ -2960,10 +2957,10 @@
         <v>12</v>
       </c>
       <c r="B46" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C46" s="6" t="s">
         <v>157</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>158</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>22</v>
@@ -2974,10 +2971,10 @@
         <v>12</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>22</v>
@@ -2988,10 +2985,10 @@
         <v>12</v>
       </c>
       <c r="B48" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C48" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>22</v>
@@ -3002,10 +2999,10 @@
         <v>12</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>163</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>22</v>
@@ -3019,7 +3016,7 @@
         <v>74</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>22</v>
@@ -3033,7 +3030,7 @@
         <v>18</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>22</v>
@@ -3047,7 +3044,7 @@
         <v>42</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>22</v>
@@ -3058,10 +3055,10 @@
         <v>16</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>22</v>
@@ -3075,7 +3072,7 @@
         <v>74</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>22</v>
@@ -3086,13 +3083,13 @@
         <v>20</v>
       </c>
       <c r="B55" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C55" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="C55" s="5" t="s">
-        <v>170</v>
-      </c>
       <c r="D55" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="56" ht="30" hidden="1" customHeight="1" spans="1:4">
@@ -3100,13 +3097,13 @@
         <v>20</v>
       </c>
       <c r="B56" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C56" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="C56" s="6" t="s">
+      <c r="D56" s="3" t="s">
         <v>172</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="57" ht="30" hidden="1" customHeight="1" spans="1:4">
@@ -3117,7 +3114,7 @@
         <v>74</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>22</v>
@@ -3128,13 +3125,13 @@
         <v>24</v>
       </c>
       <c r="B58" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C58" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="C58" s="6" t="s">
+      <c r="D58" s="3" t="s">
         <v>175</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="59" ht="30" hidden="1" customHeight="1" spans="1:4">
@@ -3142,13 +3139,13 @@
         <v>24</v>
       </c>
       <c r="B59" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C59" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="D59" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="60" ht="30" hidden="1" customHeight="1" spans="1:4">
@@ -3156,13 +3153,13 @@
         <v>24</v>
       </c>
       <c r="B60" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C60" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="D60" s="3" t="s">
         <v>181</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="61" ht="30" hidden="1" customHeight="1" spans="1:4">
@@ -3170,13 +3167,13 @@
         <v>24</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="62" ht="30" hidden="1" customHeight="1" spans="1:4">
@@ -3184,10 +3181,10 @@
         <v>24</v>
       </c>
       <c r="B62" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C62" s="6" t="s">
         <v>184</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>185</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>22</v>
@@ -3198,10 +3195,10 @@
         <v>24</v>
       </c>
       <c r="B63" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C63" s="5" t="s">
         <v>186</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>187</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>22</v>
@@ -3212,10 +3209,10 @@
         <v>24</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>22</v>
@@ -3229,7 +3226,7 @@
         <v>74</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>22</v>
@@ -3240,13 +3237,13 @@
         <v>33</v>
       </c>
       <c r="B66" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C66" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="C66" s="6" t="s">
+      <c r="D66" s="3" t="s">
         <v>191</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="67" ht="30" hidden="1" customHeight="1" spans="1:4">
@@ -3254,13 +3251,13 @@
         <v>33</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="68" ht="30" hidden="1" customHeight="1" spans="1:4">
@@ -3271,7 +3268,7 @@
         <v>35</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>22</v>
@@ -3282,10 +3279,10 @@
         <v>33</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>22</v>
@@ -3296,27 +3293,27 @@
         <v>33</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="71" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="71" ht="30" customHeight="1" spans="1:4">
       <c r="A71" t="s">
         <v>4</v>
       </c>
       <c r="B71" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D71" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="72" ht="28.8" hidden="1" spans="1:4">
@@ -3327,7 +3324,7 @@
         <v>18</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="73" hidden="1" spans="1:4">
@@ -3335,24 +3332,24 @@
         <v>59</v>
       </c>
       <c r="B73" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="74" hidden="1" spans="1:4">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
       <c r="A74" t="s">
         <v>4</v>
       </c>
       <c r="B74" t="s">
+        <v>198</v>
+      </c>
+      <c r="C74" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="C74" s="9" t="s">
+      <c r="D74" t="s">
         <v>200</v>
-      </c>
-      <c r="D74" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="75" hidden="1" spans="1:4">
@@ -3363,7 +3360,7 @@
         <v>74</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="76" hidden="1" spans="1:4">
@@ -3374,7 +3371,7 @@
         <v>52</v>
       </c>
       <c r="C76" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="77" hidden="1" spans="1:4">
@@ -3382,10 +3379,10 @@
         <v>50</v>
       </c>
       <c r="B77" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="78" hidden="1" spans="1:4">
@@ -3396,7 +3393,7 @@
         <v>74</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="79" hidden="1" spans="1:4">
@@ -3407,7 +3404,7 @@
         <v>18</v>
       </c>
       <c r="C79" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="80" hidden="1" spans="1:4">
@@ -3415,13 +3412,13 @@
         <v>59</v>
       </c>
       <c r="B80" t="s">
+        <v>206</v>
+      </c>
+      <c r="C80" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="C80" s="4" t="s">
-        <v>208</v>
-      </c>
       <c r="D80" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="81" hidden="1" spans="1:4">
@@ -3429,10 +3426,10 @@
         <v>59</v>
       </c>
       <c r="B81" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="82" hidden="1" spans="1:4">
@@ -3440,10 +3437,10 @@
         <v>59</v>
       </c>
       <c r="B82" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="83" hidden="1" spans="1:4">
@@ -3451,13 +3448,13 @@
         <v>62</v>
       </c>
       <c r="B83" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D83" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="84" hidden="1" spans="1:4">
@@ -3465,13 +3462,13 @@
         <v>62</v>
       </c>
       <c r="B84" t="s">
+        <v>211</v>
+      </c>
+      <c r="C84" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="C84" s="4" t="s">
-        <v>213</v>
-      </c>
       <c r="D84" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="85" hidden="1" spans="1:4">
@@ -3479,10 +3476,10 @@
         <v>62</v>
       </c>
       <c r="B85" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="86" hidden="1" spans="1:4">
@@ -3493,7 +3490,7 @@
         <v>74</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="87" hidden="1" spans="1:4">
@@ -3504,7 +3501,7 @@
         <v>42</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="88" hidden="1" spans="1:4">
@@ -3512,10 +3509,10 @@
         <v>65</v>
       </c>
       <c r="B88" t="s">
+        <v>214</v>
+      </c>
+      <c r="C88" s="4" t="s">
         <v>215</v>
-      </c>
-      <c r="C88" s="4" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="89" hidden="1" spans="1:4">
@@ -3523,13 +3520,13 @@
         <v>65</v>
       </c>
       <c r="B89" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D89" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="90" hidden="1" spans="1:4">
@@ -3537,165 +3534,165 @@
         <v>65</v>
       </c>
       <c r="B90" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D90" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="91" ht="72" hidden="1" spans="1:4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="91" ht="72" spans="1:4">
       <c r="A91" t="s">
         <v>4</v>
       </c>
       <c r="B91" t="s">
+        <v>218</v>
+      </c>
+      <c r="C91" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="C91" s="9" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="92" hidden="1" spans="1:4">
+    </row>
+    <row r="92" spans="1:4">
       <c r="A92" t="s">
         <v>4</v>
       </c>
       <c r="B92" t="s">
+        <v>220</v>
+      </c>
+      <c r="C92" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="C92" s="9" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4">
+    </row>
+    <row r="93" hidden="1" spans="1:4">
       <c r="A93" t="s">
         <v>68</v>
       </c>
       <c r="B93" t="s">
+        <v>222</v>
+      </c>
+      <c r="C93" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="C93" s="4" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4">
+    </row>
+    <row r="94" hidden="1" spans="1:4">
       <c r="A94" t="s">
         <v>68</v>
       </c>
       <c r="B94" t="s">
+        <v>224</v>
+      </c>
+      <c r="C94" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="C94" s="4" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4">
+    </row>
+    <row r="95" hidden="1" spans="1:4">
       <c r="A95" t="s">
         <v>68</v>
       </c>
       <c r="B95" t="s">
+        <v>226</v>
+      </c>
+      <c r="C95" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="C95" s="4" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4">
+    </row>
+    <row r="96" hidden="1" spans="1:4">
       <c r="A96" t="s">
         <v>68</v>
       </c>
       <c r="B96" t="s">
+        <v>228</v>
+      </c>
+      <c r="C96" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="C96" s="4" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4">
+    </row>
+    <row r="97" hidden="1" spans="1:4">
       <c r="A97" t="s">
         <v>68</v>
       </c>
       <c r="B97" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="98" hidden="1" spans="1:4">
       <c r="A98" t="s">
         <v>68</v>
       </c>
       <c r="B98" t="s">
+        <v>231</v>
+      </c>
+      <c r="C98" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="C98" s="4" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4">
+    </row>
+    <row r="99" hidden="1" spans="1:4">
       <c r="A99" t="s">
         <v>68</v>
       </c>
       <c r="B99" t="s">
+        <v>233</v>
+      </c>
+      <c r="C99" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="C99" s="4" t="s">
-        <v>235</v>
-      </c>
       <c r="D99" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="100" ht="28.8" spans="1:4">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="100" ht="28.8" hidden="1" spans="1:4">
       <c r="A100" t="s">
         <v>68</v>
       </c>
       <c r="B100" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C100" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D100" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="101" ht="28.8" spans="1:4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="101" ht="28.8" hidden="1" spans="1:4">
       <c r="A101" t="s">
         <v>68</v>
       </c>
       <c r="B101" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C101" s="9" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D101" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="102" hidden="1" spans="1:4">
       <c r="A102" t="s">
         <v>68</v>
       </c>
       <c r="B102" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C102" s="9" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="103" hidden="1" spans="1:4">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4">
       <c r="A103" t="s">
         <v>4</v>
       </c>
       <c r="B103" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C103" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="104" hidden="1" spans="1:4">
@@ -3703,10 +3700,10 @@
         <v>12</v>
       </c>
       <c r="B104" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C104" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="105" hidden="1" spans="1:4">
@@ -3714,10 +3711,10 @@
         <v>59</v>
       </c>
       <c r="B105" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C105" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="106" hidden="1" spans="1:4">
@@ -3725,10 +3722,10 @@
         <v>8</v>
       </c>
       <c r="B106" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C106" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="107" hidden="1" spans="1:4">
@@ -3736,10 +3733,10 @@
         <v>16</v>
       </c>
       <c r="B107" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C107" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="108" hidden="1" spans="1:4">
@@ -3747,10 +3744,10 @@
         <v>40</v>
       </c>
       <c r="B108" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C108" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="109" hidden="1" spans="1:4">
@@ -3758,17 +3755,17 @@
         <v>50</v>
       </c>
       <c r="B109" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C109" s="9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D109" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
       <filters>
-        <filter val="Projects"/>
+        <filter val="WorkOrders"/>
       </filters>
     </filterColumn>
     <extLst/>
@@ -3791,19 +3788,19 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:5">
       <c r="A1" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:5">
@@ -3811,7 +3808,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>68</v>
@@ -3820,7 +3817,7 @@
         <v>74</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:5">
@@ -3828,7 +3825,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>40</v>
@@ -3837,7 +3834,7 @@
         <v>74</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:5">
@@ -3845,7 +3842,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>59</v>
@@ -3854,7 +3851,7 @@
         <v>74</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:5">
@@ -3862,7 +3859,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>12</v>
@@ -3871,7 +3868,7 @@
         <v>74</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:5">
@@ -3879,7 +3876,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>12</v>
@@ -3888,7 +3885,7 @@
         <v>74</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:5">
@@ -3896,7 +3893,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>12</v>
@@ -3905,7 +3902,7 @@
         <v>74</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:5">
@@ -3913,7 +3910,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>50</v>
@@ -3922,7 +3919,7 @@
         <v>74</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:5">
@@ -3930,16 +3927,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:5">
@@ -3947,16 +3944,16 @@
         <v>4</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C10" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>261</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:5">
@@ -3964,16 +3961,16 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:5">
@@ -3981,7 +3978,7 @@
         <v>68</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>12</v>
@@ -3990,7 +3987,7 @@
         <v>74</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:5">
@@ -3998,7 +3995,7 @@
         <v>68</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>40</v>
@@ -4007,7 +4004,7 @@
         <v>74</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:5">
@@ -4015,7 +4012,7 @@
         <v>68</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>12</v>
@@ -4024,7 +4021,7 @@
         <v>74</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:5">
@@ -4032,7 +4029,7 @@
         <v>68</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>8</v>
@@ -4041,7 +4038,7 @@
         <v>74</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:5">
@@ -4049,7 +4046,7 @@
         <v>68</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>59</v>
@@ -4058,7 +4055,7 @@
         <v>74</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:5">
@@ -4066,7 +4063,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>12</v>
@@ -4075,7 +4072,7 @@
         <v>74</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:5">
@@ -4083,7 +4080,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>16</v>
@@ -4092,7 +4089,7 @@
         <v>74</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:5">
@@ -4100,7 +4097,7 @@
         <v>24</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>4</v>
@@ -4109,7 +4106,7 @@
         <v>74</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:5">
@@ -4117,7 +4114,7 @@
         <v>24</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>47</v>
@@ -4126,7 +4123,7 @@
         <v>74</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:5">
@@ -4134,7 +4131,7 @@
         <v>24</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>33</v>
@@ -4143,7 +4140,7 @@
         <v>74</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:5">
@@ -4151,7 +4148,7 @@
         <v>24</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>12</v>
@@ -4160,7 +4157,7 @@
         <v>74</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5">
@@ -4168,7 +4165,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>4</v>
@@ -4177,7 +4174,7 @@
         <v>74</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:5">
@@ -4185,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>12</v>
@@ -4194,7 +4191,7 @@
         <v>74</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5">
@@ -4202,7 +4199,7 @@
         <v>30</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>4</v>
@@ -4211,7 +4208,7 @@
         <v>74</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:5">
@@ -4219,7 +4216,7 @@
         <v>30</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>44</v>
@@ -4228,7 +4225,7 @@
         <v>74</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:5">
@@ -4236,16 +4233,16 @@
         <v>33</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:5">
@@ -4253,7 +4250,7 @@
         <v>33</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>68</v>
@@ -4262,7 +4259,7 @@
         <v>74</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5">
@@ -4270,7 +4267,7 @@
         <v>37</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>4</v>
@@ -4279,7 +4276,7 @@
         <v>74</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1" spans="1:5">
@@ -4287,7 +4284,7 @@
         <v>37</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>47</v>
@@ -4296,7 +4293,7 @@
         <v>74</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1" spans="1:5">
@@ -4304,7 +4301,7 @@
         <v>37</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>12</v>
@@ -4313,7 +4310,7 @@
         <v>74</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" spans="1:5">
@@ -4321,16 +4318,16 @@
         <v>8</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C32" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E32" s="3" t="s">
         <v>283</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -4338,7 +4335,7 @@
         <v>4</v>
       </c>
       <c r="B33" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C33" t="s">
         <v>59</v>
@@ -4347,7 +4344,7 @@
         <v>74</v>
       </c>
       <c r="E33" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -4355,16 +4352,16 @@
         <v>4</v>
       </c>
       <c r="B34" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C34" t="s">
+        <v>285</v>
+      </c>
+      <c r="D34" t="s">
+        <v>74</v>
+      </c>
+      <c r="E34" t="s">
         <v>286</v>
-      </c>
-      <c r="D34" t="s">
-        <v>74</v>
-      </c>
-      <c r="E34" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -4372,7 +4369,7 @@
         <v>62</v>
       </c>
       <c r="B35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C35" t="s">
         <v>16</v>
@@ -4381,7 +4378,7 @@
         <v>74</v>
       </c>
       <c r="E35" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -4389,7 +4386,7 @@
         <v>62</v>
       </c>
       <c r="B36" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C36" t="s">
         <v>59</v>
@@ -4398,7 +4395,7 @@
         <v>74</v>
       </c>
       <c r="E36" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -4406,7 +4403,7 @@
         <v>65</v>
       </c>
       <c r="B37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C37" t="s">
         <v>16</v>
@@ -4415,7 +4412,7 @@
         <v>74</v>
       </c>
       <c r="E37" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -4423,7 +4420,7 @@
         <v>65</v>
       </c>
       <c r="B38" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C38" t="s">
         <v>12</v>
@@ -4432,7 +4429,7 @@
         <v>74</v>
       </c>
       <c r="E38" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -4440,7 +4437,7 @@
         <v>68</v>
       </c>
       <c r="B39" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C39" t="s">
         <v>68</v>
@@ -4449,7 +4446,7 @@
         <v>74</v>
       </c>
       <c r="E39" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -4474,10 +4471,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>293</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -4485,10 +4482,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>294</v>
+      </c>
+      <c r="C2" t="s">
         <v>295</v>
-      </c>
-      <c r="C2" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -4496,10 +4493,10 @@
         <v>68</v>
       </c>
       <c r="B3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -4507,10 +4504,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -4518,10 +4515,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -4529,10 +4526,10 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -4540,10 +4537,10 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C7" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -4551,10 +4548,10 @@
         <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C8" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -4562,10 +4559,10 @@
         <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C9" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -4573,10 +4570,10 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -4584,10 +4581,10 @@
         <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -4595,10 +4592,10 @@
         <v>47</v>
       </c>
       <c r="B12" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C12" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -4606,10 +4603,10 @@
         <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C13" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -4617,10 +4614,10 @@
         <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -4628,10 +4625,10 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
+        <v>306</v>
+      </c>
+      <c r="C15" t="s">
         <v>307</v>
-      </c>
-      <c r="C15" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -4639,32 +4636,32 @@
         <v>37</v>
       </c>
       <c r="B16" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C16" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
+        <v>309</v>
+      </c>
+      <c r="B17" t="s">
         <v>310</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>311</v>
-      </c>
-      <c r="C17" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>312</v>
+      </c>
+      <c r="B18" t="s">
         <v>313</v>
       </c>
-      <c r="B18" t="s">
-        <v>314</v>
-      </c>
       <c r="C18" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -4672,10 +4669,10 @@
         <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -4683,10 +4680,10 @@
         <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C20" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated the meta data file
</commit_message>
<xml_diff>
--- a/python/table_metadata.xlsx
+++ b/python/table_metadata.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Triggers" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Columns!$A$1:$D$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Columns!$A$1:$D$108</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="317">
   <si>
     <t>TableName</t>
   </si>
@@ -56,7 +56,8 @@
     <t>WorkOrderNumber</t>
   </si>
   <si>
-    <t>Id is INTEGER PK for JOINs. WorkOrderNumber is TEXT never use as integer. IsDeleted=false for active. OfficeId is NULL for all records — NEVER USE OfficeId. branches = AbpOrganizationUnits table. organizations = AbpOrganizationUnits table. For location/branch/office/fort myers queries always JOIN AbpOrganizationUnits ON OrganizationId=Id and filter by DisplayName ILIKE. For count by group always use COUNT(Id) with GROUP BY. For project-wise counts use ProjectId -&gt; Projects. For phase-wise counts use PhaseId -&gt; Phases. For day-wise/daily count queries use: COUNT("WorkOrders"."Id") GROUP BY "WorkOrders"."CreationTime"::date ORDER BY date. For per-day results always cast timestamp to date using ::date. Always SELECT WorkOrderNumber and Subject for display.</t>
+    <t>NEVER SELECT Subject column — always use WorkOrderNumber for display.
+ Id is INTEGER PK for JOINs. WorkOrderNumber is TEXT never use as integer. IsDeleted=false for active. OfficeId is NULL for all records — NEVER USE OfficeId. branches = AbpOrganizationUnits table. organizations = AbpOrganizationUnits table. For location/branch/office/fort myers queries always JOIN AbpOrganizationUnits ON OrganizationId=Id and filter by DisplayName ILIKE. For count by group always use COUNT(Id) with GROUP BY. For project-wise counts use ProjectId -&gt; Projects. For phase-wise counts use PhaseId -&gt; Phases. For day-wise/daily count queries use: COUNT("WorkOrders"."Id") GROUP BY "WorkOrders"."CreationTime"::date ORDER BY date. For per-day results always cast timestamp to date using ::date. Always SELECT WorkOrderNumber and Subject for display.</t>
   </si>
   <si>
     <t>Offices</t>
@@ -263,10 +264,7 @@
     <t>Primary key INTEGER. Use in all JOINs. NOT same as WorkOrderNumber.</t>
   </si>
   <si>
-    <t>Primary display column for work orders. ALWAYS USE THIS for listing and display. Human-readable ID e.g. 08.25001260.</t>
-  </si>
-  <si>
-    <t>Human-readable TEXT ID e.g. 08.25001260. Use only for WHERE lookups by number — never as integer FK.</t>
+    <t>ALWAYS USE THIS Primary display column for work orders. ALWAYS USE THIS for listing and display. Human-readable ID e.g. 08.25001260.</t>
   </si>
   <si>
     <t>Status</t>
@@ -768,6 +766,12 @@
   </si>
   <si>
     <t>Soft delete. Always write "Phases"."IsDeleted" = false — never bare "IsDeleted"</t>
+  </si>
+  <si>
+    <t>Subject</t>
+  </si>
+  <si>
+    <t>NEVER SELECT this column. Use WorkOrderNumber for display instead.</t>
   </si>
   <si>
     <t>FromTable</t>
@@ -2367,99 +2371,99 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:4">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="C4" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:4">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>22</v>
+      <c r="C5" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:4">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="C6" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:4">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="3"/>
+      <c r="C7" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:4">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:4">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="B9" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>90</v>
-      </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:4">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>90</v>
+      <c r="C10" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:4">
@@ -2467,27 +2471,27 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:4">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>97</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:4">
@@ -2495,26 +2499,26 @@
         <v>4</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>100</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:4">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="C14" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -2523,26 +2527,26 @@
         <v>4</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:4">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="C16" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>22</v>
       </c>
     </row>
@@ -2551,804 +2555,801 @@
         <v>4</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:4">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C18" s="3" t="s">
+      <c r="B18" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="C18" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:4">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1" spans="1:4">
-      <c r="A20" s="3" t="s">
+      <c r="C19" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A21" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A22" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A23" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="24" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A24" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A25" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A26" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="27" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A27" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="28" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A28" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A29" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A31" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A33" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A35" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A37" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A38" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="39" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A39" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A40" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A41" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A43" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="44" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A44" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="45" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A45" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="46" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="47" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A47" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="48" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="49" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A49" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="50" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A50" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="51" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A51" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="52" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A52" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="53" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A53" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="54" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A54" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="55" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A55" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="56" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A56" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="57" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A57" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="58" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A58" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="59" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A59" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="60" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A60" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="61" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A61" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="62" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A62" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="63" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A63" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="64" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A64" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="65" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A65" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="66" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A66" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="67" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A67" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="68" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A68" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="69" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A69" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1" spans="1:4">
+      <c r="A70" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="21" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A21" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A22" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A23" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A24" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="25" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A25" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="B70" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="26" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A26" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="C26" s="6" t="s">
+      <c r="C70" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="D70" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="27" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A27" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="28" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A28" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="29" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A29" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="30" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A30" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="31" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A31" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A32" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="33" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A33" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B33" s="2" t="s">
+    </row>
+    <row r="71" ht="28.8" hidden="1" spans="1:4">
+      <c r="A71" t="s">
+        <v>59</v>
+      </c>
+      <c r="B71" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="34" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A34" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="35" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A35" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="36" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A36" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="37" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A37" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="38" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A38" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="39" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A39" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="40" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A40" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="41" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A41" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="42" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A42" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="43" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A43" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="44" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A44" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="45" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A45" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="46" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A46" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="47" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="48" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A48" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="49" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="50" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A50" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="51" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A51" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="52" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A52" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="53" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A53" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="54" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A54" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="55" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A55" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C55" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="56" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A56" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="57" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A57" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="58" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A58" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="59" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A59" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="60" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A60" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="61" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A61" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="62" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A62" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="63" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A63" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="64" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A64" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="65" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A65" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C65" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="66" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A66" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="67" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A67" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C67" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="68" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A68" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="69" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A69" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C69" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="70" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A70" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="71" ht="30" customHeight="1" spans="1:4">
-      <c r="A71" t="s">
-        <v>4</v>
-      </c>
-      <c r="B71" t="s">
-        <v>122</v>
-      </c>
-      <c r="C71" s="7" t="s">
+      <c r="C71" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="D71" s="12" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="72" ht="28.8" hidden="1" spans="1:4">
+    </row>
+    <row r="72" hidden="1" spans="1:4">
       <c r="A72" t="s">
         <v>59</v>
       </c>
       <c r="B72" t="s">
-        <v>18</v>
-      </c>
-      <c r="C72" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C72" s="4" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="73" hidden="1" spans="1:4">
+    <row r="73" spans="1:4">
       <c r="A73" t="s">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="B73" t="s">
-        <v>137</v>
-      </c>
-      <c r="C73" s="4" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="74" spans="1:4">
+      <c r="C73" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="D73" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="74" hidden="1" spans="1:4">
       <c r="A74" t="s">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="B74" t="s">
-        <v>198</v>
-      </c>
-      <c r="C74" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="D74" t="s">
+        <v>74</v>
+      </c>
+      <c r="C74" s="4" t="s">
         <v>200</v>
       </c>
     </row>
@@ -3357,9 +3358,9 @@
         <v>50</v>
       </c>
       <c r="B75" t="s">
-        <v>74</v>
-      </c>
-      <c r="C75" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C75" s="9" t="s">
         <v>201</v>
       </c>
     </row>
@@ -3368,18 +3369,18 @@
         <v>50</v>
       </c>
       <c r="B76" t="s">
-        <v>52</v>
-      </c>
-      <c r="C76" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C76" s="4" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="77" hidden="1" spans="1:4">
       <c r="A77" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="B77" t="s">
-        <v>130</v>
+        <v>74</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>203</v>
@@ -3390,9 +3391,9 @@
         <v>59</v>
       </c>
       <c r="B78" t="s">
-        <v>74</v>
-      </c>
-      <c r="C78" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C78" s="9" t="s">
         <v>204</v>
       </c>
     </row>
@@ -3401,10 +3402,13 @@
         <v>59</v>
       </c>
       <c r="B79" t="s">
-        <v>18</v>
-      </c>
-      <c r="C79" s="9" t="s">
         <v>205</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="D79" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="80" hidden="1" spans="1:4">
@@ -3412,13 +3416,10 @@
         <v>59</v>
       </c>
       <c r="B80" t="s">
-        <v>206</v>
+        <v>136</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>207</v>
-      </c>
-      <c r="D80" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="81" hidden="1" spans="1:4">
@@ -3426,7 +3427,7 @@
         <v>59</v>
       </c>
       <c r="B81" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>208</v>
@@ -3434,13 +3435,16 @@
     </row>
     <row r="82" hidden="1" spans="1:4">
       <c r="A82" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B82" t="s">
-        <v>130</v>
+        <v>169</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>209</v>
+      </c>
+      <c r="D82" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="83" hidden="1" spans="1:4">
@@ -3448,13 +3452,13 @@
         <v>62</v>
       </c>
       <c r="B83" t="s">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D83" t="s">
-        <v>172</v>
+        <v>123</v>
       </c>
     </row>
     <row r="84" hidden="1" spans="1:4">
@@ -3462,24 +3466,21 @@
         <v>62</v>
       </c>
       <c r="B84" t="s">
-        <v>211</v>
+        <v>129</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="D84" t="s">
-        <v>124</v>
+        <v>186</v>
       </c>
     </row>
     <row r="85" hidden="1" spans="1:4">
       <c r="A85" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B85" t="s">
-        <v>130</v>
+        <v>74</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>187</v>
+        <v>166</v>
       </c>
     </row>
     <row r="86" hidden="1" spans="1:4">
@@ -3487,10 +3488,10 @@
         <v>65</v>
       </c>
       <c r="B86" t="s">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
     </row>
     <row r="87" hidden="1" spans="1:4">
@@ -3498,10 +3499,10 @@
         <v>65</v>
       </c>
       <c r="B87" t="s">
-        <v>42</v>
+        <v>213</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="88" hidden="1" spans="1:4">
@@ -3509,10 +3510,13 @@
         <v>65</v>
       </c>
       <c r="B88" t="s">
-        <v>214</v>
+        <v>169</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>215</v>
+      </c>
+      <c r="D88" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="89" hidden="1" spans="1:4">
@@ -3520,49 +3524,46 @@
         <v>65</v>
       </c>
       <c r="B89" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>216</v>
       </c>
       <c r="D89" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="90" hidden="1" spans="1:4">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="90" ht="72" spans="1:4">
       <c r="A90" t="s">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="B90" t="s">
-        <v>168</v>
-      </c>
-      <c r="C90" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="D90" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="91" ht="72" spans="1:4">
+      <c r="C90" s="9" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
       <c r="A91" t="s">
         <v>4</v>
       </c>
       <c r="B91" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C91" s="9" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="92" hidden="1" spans="1:4">
       <c r="A92" t="s">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="B92" t="s">
-        <v>220</v>
-      </c>
-      <c r="C92" s="9" t="s">
         <v>221</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="93" hidden="1" spans="1:4">
@@ -3570,10 +3571,10 @@
         <v>68</v>
       </c>
       <c r="B93" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="94" hidden="1" spans="1:4">
@@ -3581,10 +3582,10 @@
         <v>68</v>
       </c>
       <c r="B94" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="95" hidden="1" spans="1:4">
@@ -3592,10 +3593,10 @@
         <v>68</v>
       </c>
       <c r="B95" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="96" hidden="1" spans="1:4">
@@ -3603,7 +3604,7 @@
         <v>68</v>
       </c>
       <c r="B96" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="C96" s="4" t="s">
         <v>229</v>
@@ -3614,10 +3615,10 @@
         <v>68</v>
       </c>
       <c r="B97" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="98" hidden="1" spans="1:4">
@@ -3625,24 +3626,27 @@
         <v>68</v>
       </c>
       <c r="B98" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="99" hidden="1" spans="1:4">
+        <v>233</v>
+      </c>
+      <c r="D98" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="99" ht="28.8" hidden="1" spans="1:4">
       <c r="A99" t="s">
         <v>68</v>
       </c>
       <c r="B99" t="s">
-        <v>233</v>
-      </c>
-      <c r="C99" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C99" s="9" t="s">
         <v>234</v>
       </c>
       <c r="D99" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
     </row>
     <row r="100" ht="28.8" hidden="1" spans="1:4">
@@ -3650,46 +3654,43 @@
         <v>68</v>
       </c>
       <c r="B100" t="s">
-        <v>125</v>
+        <v>87</v>
       </c>
       <c r="C100" s="9" t="s">
         <v>235</v>
       </c>
       <c r="D100" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="101" ht="28.8" hidden="1" spans="1:4">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="101" hidden="1" spans="1:4">
       <c r="A101" t="s">
         <v>68</v>
       </c>
       <c r="B101" t="s">
-        <v>88</v>
+        <v>129</v>
       </c>
       <c r="C101" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="D101" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="102" hidden="1" spans="1:4">
+    </row>
+    <row r="102" spans="1:4">
       <c r="A102" t="s">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="B102" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C102" s="9" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="103" spans="1:4">
+    <row r="103" hidden="1" spans="1:4">
       <c r="A103" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B103" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C103" s="9" t="s">
         <v>238</v>
@@ -3697,10 +3698,10 @@
     </row>
     <row r="104" hidden="1" spans="1:4">
       <c r="A104" t="s">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="B104" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C104" s="9" t="s">
         <v>239</v>
@@ -3708,10 +3709,10 @@
     </row>
     <row r="105" hidden="1" spans="1:4">
       <c r="A105" t="s">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="B105" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C105" s="9" t="s">
         <v>240</v>
@@ -3719,10 +3720,10 @@
     </row>
     <row r="106" hidden="1" spans="1:4">
       <c r="A106" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="B106" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C106" s="9" t="s">
         <v>241</v>
@@ -3730,10 +3731,10 @@
     </row>
     <row r="107" hidden="1" spans="1:4">
       <c r="A107" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B107" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C107" s="9" t="s">
         <v>242</v>
@@ -3741,28 +3742,28 @@
     </row>
     <row r="108" hidden="1" spans="1:4">
       <c r="A108" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B108" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C108" s="9" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="109" hidden="1" spans="1:4">
+    <row r="109" spans="1:4">
       <c r="A109" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="B109" t="s">
-        <v>130</v>
-      </c>
-      <c r="C109" s="9" t="s">
         <v>244</v>
       </c>
+      <c r="C109" t="s">
+        <v>245</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D109" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D108" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
       <filters>
         <filter val="WorkOrders"/>
@@ -3788,19 +3789,19 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:5">
@@ -3808,7 +3809,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>68</v>
@@ -3817,7 +3818,7 @@
         <v>74</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:5">
@@ -3825,7 +3826,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>40</v>
@@ -3834,7 +3835,7 @@
         <v>74</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:5">
@@ -3842,7 +3843,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>59</v>
@@ -3851,7 +3852,7 @@
         <v>74</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:5">
@@ -3859,7 +3860,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>12</v>
@@ -3868,7 +3869,7 @@
         <v>74</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:5">
@@ -3876,7 +3877,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>12</v>
@@ -3885,7 +3886,7 @@
         <v>74</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:5">
@@ -3893,7 +3894,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>12</v>
@@ -3902,7 +3903,7 @@
         <v>74</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:5">
@@ -3910,7 +3911,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>50</v>
@@ -3919,7 +3920,7 @@
         <v>74</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:5">
@@ -3927,16 +3928,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:5">
@@ -3944,16 +3945,16 @@
         <v>4</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:5">
@@ -3961,16 +3962,16 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:5">
@@ -3978,7 +3979,7 @@
         <v>68</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>12</v>
@@ -3987,7 +3988,7 @@
         <v>74</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:5">
@@ -3995,7 +3996,7 @@
         <v>68</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>40</v>
@@ -4004,7 +4005,7 @@
         <v>74</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:5">
@@ -4012,7 +4013,7 @@
         <v>68</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>12</v>
@@ -4021,7 +4022,7 @@
         <v>74</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:5">
@@ -4029,7 +4030,7 @@
         <v>68</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>8</v>
@@ -4038,7 +4039,7 @@
         <v>74</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:5">
@@ -4046,7 +4047,7 @@
         <v>68</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>59</v>
@@ -4055,7 +4056,7 @@
         <v>74</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:5">
@@ -4063,7 +4064,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>12</v>
@@ -4072,7 +4073,7 @@
         <v>74</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:5">
@@ -4080,7 +4081,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>16</v>
@@ -4089,7 +4090,7 @@
         <v>74</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:5">
@@ -4097,7 +4098,7 @@
         <v>24</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>4</v>
@@ -4106,7 +4107,7 @@
         <v>74</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:5">
@@ -4114,7 +4115,7 @@
         <v>24</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>47</v>
@@ -4123,7 +4124,7 @@
         <v>74</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:5">
@@ -4131,7 +4132,7 @@
         <v>24</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>33</v>
@@ -4140,7 +4141,7 @@
         <v>74</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:5">
@@ -4148,7 +4149,7 @@
         <v>24</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>12</v>
@@ -4157,7 +4158,7 @@
         <v>74</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5">
@@ -4165,7 +4166,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>4</v>
@@ -4174,7 +4175,7 @@
         <v>74</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:5">
@@ -4182,7 +4183,7 @@
         <v>27</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>12</v>
@@ -4191,7 +4192,7 @@
         <v>74</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5">
@@ -4199,7 +4200,7 @@
         <v>30</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>4</v>
@@ -4208,7 +4209,7 @@
         <v>74</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:5">
@@ -4216,7 +4217,7 @@
         <v>30</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>44</v>
@@ -4225,7 +4226,7 @@
         <v>74</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:5">
@@ -4233,16 +4234,16 @@
         <v>33</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:5">
@@ -4250,7 +4251,7 @@
         <v>33</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>68</v>
@@ -4259,7 +4260,7 @@
         <v>74</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5">
@@ -4267,7 +4268,7 @@
         <v>37</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>4</v>
@@ -4276,7 +4277,7 @@
         <v>74</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1" spans="1:5">
@@ -4284,7 +4285,7 @@
         <v>37</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>47</v>
@@ -4293,7 +4294,7 @@
         <v>74</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1" spans="1:5">
@@ -4301,7 +4302,7 @@
         <v>37</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>12</v>
@@ -4310,7 +4311,7 @@
         <v>74</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" spans="1:5">
@@ -4318,16 +4319,16 @@
         <v>8</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -4335,7 +4336,7 @@
         <v>4</v>
       </c>
       <c r="B33" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C33" t="s">
         <v>59</v>
@@ -4344,7 +4345,7 @@
         <v>74</v>
       </c>
       <c r="E33" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -4352,16 +4353,16 @@
         <v>4</v>
       </c>
       <c r="B34" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C34" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D34" t="s">
         <v>74</v>
       </c>
       <c r="E34" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -4369,7 +4370,7 @@
         <v>62</v>
       </c>
       <c r="B35" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C35" t="s">
         <v>16</v>
@@ -4378,7 +4379,7 @@
         <v>74</v>
       </c>
       <c r="E35" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -4386,7 +4387,7 @@
         <v>62</v>
       </c>
       <c r="B36" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C36" t="s">
         <v>59</v>
@@ -4395,7 +4396,7 @@
         <v>74</v>
       </c>
       <c r="E36" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -4403,7 +4404,7 @@
         <v>65</v>
       </c>
       <c r="B37" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C37" t="s">
         <v>16</v>
@@ -4412,7 +4413,7 @@
         <v>74</v>
       </c>
       <c r="E37" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -4420,7 +4421,7 @@
         <v>65</v>
       </c>
       <c r="B38" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C38" t="s">
         <v>12</v>
@@ -4429,7 +4430,7 @@
         <v>74</v>
       </c>
       <c r="E38" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -4437,7 +4438,7 @@
         <v>68</v>
       </c>
       <c r="B39" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C39" t="s">
         <v>68</v>
@@ -4446,7 +4447,7 @@
         <v>74</v>
       </c>
       <c r="E39" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -4471,10 +4472,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -4482,10 +4483,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -4493,10 +4494,10 @@
         <v>68</v>
       </c>
       <c r="B3" t="s">
+        <v>297</v>
+      </c>
+      <c r="C3" t="s">
         <v>296</v>
-      </c>
-      <c r="C3" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -4504,10 +4505,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C4" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -4515,10 +4516,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -4526,10 +4527,10 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -4537,10 +4538,10 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -4548,10 +4549,10 @@
         <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -4559,10 +4560,10 @@
         <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -4570,10 +4571,10 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -4581,10 +4582,10 @@
         <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -4592,10 +4593,10 @@
         <v>47</v>
       </c>
       <c r="B12" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C12" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -4603,10 +4604,10 @@
         <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C13" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -4614,10 +4615,10 @@
         <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -4625,10 +4626,10 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C15" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -4636,32 +4637,32 @@
         <v>37</v>
       </c>
       <c r="B16" t="s">
+        <v>309</v>
+      </c>
+      <c r="C16" t="s">
         <v>308</v>
-      </c>
-      <c r="C16" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B17" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C17" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>313</v>
+      </c>
+      <c r="B18" t="s">
+        <v>314</v>
+      </c>
+      <c r="C18" t="s">
         <v>312</v>
-      </c>
-      <c r="B18" t="s">
-        <v>313</v>
-      </c>
-      <c r="C18" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -4669,10 +4670,10 @@
         <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C19" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -4680,10 +4681,10 @@
         <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C20" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemented the chart details in tables
</commit_message>
<xml_diff>
--- a/python/table_metadata.xlsx
+++ b/python/table_metadata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9840" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="9840" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Triggers" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Columns!$A$1:$D$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Columns!$A$1:$D$109</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="318">
   <si>
     <t>TableName</t>
   </si>
@@ -57,7 +57,15 @@
   </si>
   <si>
     <t>NEVER SELECT Subject column — always use WorkOrderNumber for display.
- Id is INTEGER PK for JOINs. WorkOrderNumber is TEXT never use as integer. IsDeleted=false for active. OfficeId is NULL for all records — NEVER USE OfficeId. branches = AbpOrganizationUnits table. organizations = AbpOrganizationUnits table. For location/branch/office/fort myers queries always JOIN AbpOrganizationUnits ON OrganizationId=Id and filter by DisplayName ILIKE. For count by group always use COUNT(Id) with GROUP BY. For project-wise counts use ProjectId -&gt; Projects. For phase-wise counts use PhaseId -&gt; Phases. For day-wise/daily count queries use: COUNT("WorkOrders"."Id") GROUP BY "WorkOrders"."CreationTime"::date ORDER BY date. For per-day results always cast timestamp to date using ::date. Always SELECT WorkOrderNumber and Subject for display.</t>
+ Id is INTEGER PK for JOINs. WorkOrderNumber is TEXT never use as integer. IsDeleted=false for active. 
+ OfficeId is NULL for all records — NEVER USE OfficeId. branches = AbpOrganizationUnits table. 
+ organizations = AbpOrganizationUnits table. For location/branch/office/fort myers queries always 
+ JOIN AbpOrganizationUnits ON OrganizationId=Id and filter by DisplayName ILIKE. For count by group 
+ always use COUNT(Id) with GROUP BY. For project-wise counts use ProjectId -&gt; Projects. For phase-wise
+ counts use PhaseId -&gt; Phases. For day-wise/daily count queries use: COUNT("WorkOrders"."Id") GROUP
+ BY "WorkOrders"."CreationTime"::date ORDER BY date. For per-day results always cast timestamp to 
+ date using ::date. Always SELECT WorkOrderNumber for display — NEVER SELECT Subject. Office names come 
+ from AbpOrganizationUnits.DisplayName via OrganizationId — NOT from Offices table..</t>
   </si>
   <si>
     <t>Offices</t>
@@ -930,7 +938,7 @@
     <t>project,projects</t>
   </si>
   <si>
-    <t>organization,organizations,org,unit,units,branch,branches,location</t>
+    <t>office,offices</t>
   </si>
   <si>
     <t>user,users,username,creator,created,technician,active</t>
@@ -940,6 +948,9 @@
   </si>
   <si>
     <t>phase,phases</t>
+  </si>
+  <si>
+    <t>organization,organizations,org,unit,units,branch,branches,location,office,offices,officename</t>
   </si>
   <si>
     <t>specimen,sample,test,tests</t>
@@ -1635,6 +1646,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1653,9 +1667,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="distributed"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2014,9 +2025,9 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="65" style="9" customWidth="1"/>
+    <col min="2" max="2" width="65" style="10" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="70" style="9" customWidth="1"/>
+    <col min="4" max="4" width="70" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:4">
@@ -2034,240 +2045,240 @@
       </c>
     </row>
     <row r="2" s="10" customFormat="1" ht="144" customHeight="1" spans="1:4">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" ht="64" customHeight="1" spans="1:4">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:4">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:4">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:4">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="C6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:4">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="C7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:4">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="C8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:4">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="C9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:4">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:4">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="C11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:4">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:4">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="3" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:4">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="4" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:4">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:4">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:4">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="3" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:4">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="4" t="s">
         <v>61</v>
       </c>
     </row>
@@ -2275,10 +2286,10 @@
       <c r="A19" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="10" t="s">
         <v>64</v>
       </c>
     </row>
@@ -2286,13 +2297,13 @@
       <c r="A20" t="s">
         <v>65</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C20" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="10" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2300,13 +2311,13 @@
       <c r="A21" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="10" t="s">
         <v>69</v>
       </c>
       <c r="C21" t="s">
         <v>70</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="10" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2324,7 +2335,7 @@
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="81.8888888888889" style="4" customWidth="1"/>
+    <col min="3" max="3" width="81.8888888888889" style="5" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2343,952 +2354,952 @@
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:4">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:4">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:4">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:4">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:4">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="4"/>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:4">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:4">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:4">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:4">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:4">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:4">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:4">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:4">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:4">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:4">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:4">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:4">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:4">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="20" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="5" t="s">
+      <c r="B20" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="21" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="22" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="23" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="4" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="24" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="3" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="25" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="4" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="26" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="3" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="27" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="4" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="28" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="29" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="30" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C30" s="5" t="s">
+      <c r="B30" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="31" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="32" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="33" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="34" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="35" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="36" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="D36" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="37" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A37" s="3" t="s">
+      <c r="A37" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="38" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="D38" s="3" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="39" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="40" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C40" s="5" t="s">
+      <c r="B40" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="D40" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="41" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="D42" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="43" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="44" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A44" s="2" t="s">
+      <c r="A44" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="D44" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="45" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="D45" s="3" t="s">
+      <c r="D45" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="46" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A46" s="2" t="s">
+      <c r="A46" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="D46" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="47" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B47" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="D47" s="3" t="s">
+      <c r="D47" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="48" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A48" s="2" t="s">
+      <c r="A48" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="C48" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="D48" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="49" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B49" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C49" s="6" t="s">
+      <c r="B49" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C49" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="D49" s="3" t="s">
+      <c r="D49" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="50" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A50" s="2" t="s">
+      <c r="A50" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C50" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="D50" s="2" t="s">
+      <c r="D50" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="51" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="B51" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="D51" s="3" t="s">
+      <c r="D51" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="52" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A52" s="2" t="s">
+      <c r="A52" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C52" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="D52" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="53" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A53" s="3" t="s">
+      <c r="A53" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B53" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C53" s="6" t="s">
+      <c r="B53" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C53" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D53" s="3" t="s">
+      <c r="D53" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="54" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A54" s="2" t="s">
+      <c r="A54" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="D54" s="3" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="55" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B55" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C55" s="6" t="s">
+      <c r="C55" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="D55" s="4" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="56" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A56" s="2" t="s">
+      <c r="A56" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C56" s="5" t="s">
+      <c r="B56" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C56" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="D56" s="2" t="s">
+      <c r="D56" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="57" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A57" s="3" t="s">
+      <c r="A57" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B57" s="3" t="s">
+      <c r="B57" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C57" s="6" t="s">
+      <c r="C57" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="D57" s="3" t="s">
+      <c r="D57" s="4" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="58" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A58" s="2" t="s">
+      <c r="A58" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="C58" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="D58" s="3" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="59" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A59" s="3" t="s">
+      <c r="A59" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B59" s="3" t="s">
+      <c r="B59" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="D59" s="3" t="s">
+      <c r="D59" s="4" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="60" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A60" s="2" t="s">
+      <c r="A60" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="C60" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="D60" s="2" t="s">
+      <c r="D60" s="3" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="61" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A61" s="3" t="s">
+      <c r="A61" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="B61" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="C61" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="D61" s="3" t="s">
+      <c r="D61" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="62" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A62" s="2" t="s">
+      <c r="A62" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="C62" s="5" t="s">
+      <c r="C62" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="D62" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="63" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A63" s="3" t="s">
+      <c r="A63" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="B63" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C63" s="6" t="s">
+      <c r="C63" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="D63" s="3" t="s">
+      <c r="D63" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="64" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A64" s="2" t="s">
+      <c r="A64" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B64" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C64" s="5" t="s">
+      <c r="B64" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C64" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="D64" s="2" t="s">
+      <c r="D64" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="65" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B65" s="3" t="s">
+      <c r="B65" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="C65" s="6" t="s">
+      <c r="C65" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="D65" s="3" t="s">
+      <c r="D65" s="4" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="66" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A66" s="2" t="s">
+      <c r="A66" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C66" s="5" t="s">
+      <c r="C66" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="D66" s="3" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="67" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A67" s="3" t="s">
+      <c r="A67" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B67" s="3" t="s">
+      <c r="B67" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C67" s="6" t="s">
+      <c r="C67" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="D67" s="3" t="s">
+      <c r="D67" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="68" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A68" s="2" t="s">
+      <c r="A68" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C68" s="5" t="s">
+      <c r="C68" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="D68" s="2" t="s">
+      <c r="D68" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="69" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A69" s="3" t="s">
+      <c r="A69" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B69" s="3" t="s">
+      <c r="B69" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C69" s="6" t="s">
+      <c r="C69" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="D69" s="3" t="s">
+      <c r="D69" s="4" t="s">
         <v>22</v>
       </c>
     </row>
@@ -3299,7 +3310,7 @@
       <c r="B70" t="s">
         <v>121</v>
       </c>
-      <c r="C70" s="7" t="s">
+      <c r="C70" s="8" t="s">
         <v>194</v>
       </c>
       <c r="D70" s="12" t="s">
@@ -3313,7 +3324,7 @@
       <c r="B71" t="s">
         <v>18</v>
       </c>
-      <c r="C71" s="8" t="s">
+      <c r="C71" s="9" t="s">
         <v>195</v>
       </c>
     </row>
@@ -3324,7 +3335,7 @@
       <c r="B72" t="s">
         <v>136</v>
       </c>
-      <c r="C72" s="4" t="s">
+      <c r="C72" s="5" t="s">
         <v>196</v>
       </c>
     </row>
@@ -3335,7 +3346,7 @@
       <c r="B73" t="s">
         <v>197</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="10" t="s">
         <v>198</v>
       </c>
       <c r="D73" t="s">
@@ -3349,7 +3360,7 @@
       <c r="B74" t="s">
         <v>74</v>
       </c>
-      <c r="C74" s="4" t="s">
+      <c r="C74" s="5" t="s">
         <v>200</v>
       </c>
     </row>
@@ -3360,7 +3371,7 @@
       <c r="B75" t="s">
         <v>52</v>
       </c>
-      <c r="C75" s="9" t="s">
+      <c r="C75" s="10" t="s">
         <v>201</v>
       </c>
     </row>
@@ -3371,7 +3382,7 @@
       <c r="B76" t="s">
         <v>129</v>
       </c>
-      <c r="C76" s="4" t="s">
+      <c r="C76" s="5" t="s">
         <v>202</v>
       </c>
     </row>
@@ -3382,7 +3393,7 @@
       <c r="B77" t="s">
         <v>74</v>
       </c>
-      <c r="C77" s="4" t="s">
+      <c r="C77" s="5" t="s">
         <v>203</v>
       </c>
     </row>
@@ -3393,7 +3404,7 @@
       <c r="B78" t="s">
         <v>18</v>
       </c>
-      <c r="C78" s="9" t="s">
+      <c r="C78" s="10" t="s">
         <v>204</v>
       </c>
     </row>
@@ -3404,7 +3415,7 @@
       <c r="B79" t="s">
         <v>205</v>
       </c>
-      <c r="C79" s="4" t="s">
+      <c r="C79" s="5" t="s">
         <v>206</v>
       </c>
       <c r="D79" t="s">
@@ -3418,7 +3429,7 @@
       <c r="B80" t="s">
         <v>136</v>
       </c>
-      <c r="C80" s="4" t="s">
+      <c r="C80" s="5" t="s">
         <v>207</v>
       </c>
     </row>
@@ -3429,7 +3440,7 @@
       <c r="B81" t="s">
         <v>129</v>
       </c>
-      <c r="C81" s="4" t="s">
+      <c r="C81" s="5" t="s">
         <v>208</v>
       </c>
     </row>
@@ -3440,7 +3451,7 @@
       <c r="B82" t="s">
         <v>169</v>
       </c>
-      <c r="C82" s="4" t="s">
+      <c r="C82" s="5" t="s">
         <v>209</v>
       </c>
       <c r="D82" t="s">
@@ -3454,7 +3465,7 @@
       <c r="B83" t="s">
         <v>210</v>
       </c>
-      <c r="C83" s="4" t="s">
+      <c r="C83" s="5" t="s">
         <v>211</v>
       </c>
       <c r="D83" t="s">
@@ -3468,7 +3479,7 @@
       <c r="B84" t="s">
         <v>129</v>
       </c>
-      <c r="C84" s="4" t="s">
+      <c r="C84" s="5" t="s">
         <v>186</v>
       </c>
     </row>
@@ -3479,7 +3490,7 @@
       <c r="B85" t="s">
         <v>74</v>
       </c>
-      <c r="C85" s="4" t="s">
+      <c r="C85" s="5" t="s">
         <v>166</v>
       </c>
     </row>
@@ -3490,7 +3501,7 @@
       <c r="B86" t="s">
         <v>42</v>
       </c>
-      <c r="C86" s="4" t="s">
+      <c r="C86" s="5" t="s">
         <v>212</v>
       </c>
     </row>
@@ -3501,7 +3512,7 @@
       <c r="B87" t="s">
         <v>213</v>
       </c>
-      <c r="C87" s="4" t="s">
+      <c r="C87" s="5" t="s">
         <v>214</v>
       </c>
     </row>
@@ -3512,7 +3523,7 @@
       <c r="B88" t="s">
         <v>169</v>
       </c>
-      <c r="C88" s="4" t="s">
+      <c r="C88" s="5" t="s">
         <v>215</v>
       </c>
       <c r="D88" t="s">
@@ -3526,7 +3537,7 @@
       <c r="B89" t="s">
         <v>167</v>
       </c>
-      <c r="C89" s="4" t="s">
+      <c r="C89" s="5" t="s">
         <v>216</v>
       </c>
       <c r="D89" t="s">
@@ -3540,7 +3551,7 @@
       <c r="B90" t="s">
         <v>217</v>
       </c>
-      <c r="C90" s="9" t="s">
+      <c r="C90" s="10" t="s">
         <v>218</v>
       </c>
     </row>
@@ -3551,7 +3562,7 @@
       <c r="B91" t="s">
         <v>219</v>
       </c>
-      <c r="C91" s="9" t="s">
+      <c r="C91" s="10" t="s">
         <v>220</v>
       </c>
     </row>
@@ -3562,7 +3573,7 @@
       <c r="B92" t="s">
         <v>221</v>
       </c>
-      <c r="C92" s="4" t="s">
+      <c r="C92" s="5" t="s">
         <v>222</v>
       </c>
     </row>
@@ -3573,7 +3584,7 @@
       <c r="B93" t="s">
         <v>223</v>
       </c>
-      <c r="C93" s="4" t="s">
+      <c r="C93" s="5" t="s">
         <v>224</v>
       </c>
     </row>
@@ -3584,7 +3595,7 @@
       <c r="B94" t="s">
         <v>225</v>
       </c>
-      <c r="C94" s="4" t="s">
+      <c r="C94" s="5" t="s">
         <v>226</v>
       </c>
     </row>
@@ -3595,7 +3606,7 @@
       <c r="B95" t="s">
         <v>227</v>
       </c>
-      <c r="C95" s="4" t="s">
+      <c r="C95" s="5" t="s">
         <v>228</v>
       </c>
     </row>
@@ -3606,7 +3617,7 @@
       <c r="B96" t="s">
         <v>217</v>
       </c>
-      <c r="C96" s="4" t="s">
+      <c r="C96" s="5" t="s">
         <v>229</v>
       </c>
     </row>
@@ -3617,7 +3628,7 @@
       <c r="B97" t="s">
         <v>230</v>
       </c>
-      <c r="C97" s="4" t="s">
+      <c r="C97" s="5" t="s">
         <v>231</v>
       </c>
     </row>
@@ -3628,7 +3639,7 @@
       <c r="B98" t="s">
         <v>232</v>
       </c>
-      <c r="C98" s="4" t="s">
+      <c r="C98" s="5" t="s">
         <v>233</v>
       </c>
       <c r="D98" t="s">
@@ -3642,7 +3653,7 @@
       <c r="B99" t="s">
         <v>124</v>
       </c>
-      <c r="C99" s="9" t="s">
+      <c r="C99" s="10" t="s">
         <v>234</v>
       </c>
       <c r="D99" t="s">
@@ -3656,7 +3667,7 @@
       <c r="B100" t="s">
         <v>87</v>
       </c>
-      <c r="C100" s="9" t="s">
+      <c r="C100" s="10" t="s">
         <v>235</v>
       </c>
       <c r="D100" t="s">
@@ -3670,7 +3681,7 @@
       <c r="B101" t="s">
         <v>129</v>
       </c>
-      <c r="C101" s="9" t="s">
+      <c r="C101" s="10" t="s">
         <v>236</v>
       </c>
     </row>
@@ -3681,7 +3692,7 @@
       <c r="B102" t="s">
         <v>129</v>
       </c>
-      <c r="C102" s="9" t="s">
+      <c r="C102" s="10" t="s">
         <v>237</v>
       </c>
     </row>
@@ -3692,7 +3703,7 @@
       <c r="B103" t="s">
         <v>129</v>
       </c>
-      <c r="C103" s="9" t="s">
+      <c r="C103" s="10" t="s">
         <v>238</v>
       </c>
     </row>
@@ -3703,7 +3714,7 @@
       <c r="B104" t="s">
         <v>129</v>
       </c>
-      <c r="C104" s="9" t="s">
+      <c r="C104" s="10" t="s">
         <v>239</v>
       </c>
     </row>
@@ -3714,7 +3725,7 @@
       <c r="B105" t="s">
         <v>129</v>
       </c>
-      <c r="C105" s="9" t="s">
+      <c r="C105" s="10" t="s">
         <v>240</v>
       </c>
     </row>
@@ -3725,7 +3736,7 @@
       <c r="B106" t="s">
         <v>129</v>
       </c>
-      <c r="C106" s="9" t="s">
+      <c r="C106" s="10" t="s">
         <v>241</v>
       </c>
     </row>
@@ -3736,7 +3747,7 @@
       <c r="B107" t="s">
         <v>129</v>
       </c>
-      <c r="C107" s="9" t="s">
+      <c r="C107" s="10" t="s">
         <v>242</v>
       </c>
     </row>
@@ -3747,7 +3758,7 @@
       <c r="B108" t="s">
         <v>129</v>
       </c>
-      <c r="C108" s="9" t="s">
+      <c r="C108" s="10" t="s">
         <v>243</v>
       </c>
     </row>
@@ -3763,11 +3774,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D108" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D109" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
-      <filters>
-        <filter val="WorkOrders"/>
-      </filters>
+      <customFilters>
+        <customFilter operator="equal" val="WorkOrders"/>
+      </customFilters>
     </filterColumn>
     <extLst/>
   </autoFilter>
@@ -3805,529 +3816,529 @@
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:5">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="D2" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:5">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="D3" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:5">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="D4" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:5">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="D5" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:5">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="D6" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:5">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="D7" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:5">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E8" s="3" t="s">
+      <c r="D8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:5">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" s="2" t="s">
+      <c r="D9" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:5">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E10" s="3" t="s">
+      <c r="D10" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:5">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="D11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:5">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E12" s="3" t="s">
+      <c r="D12" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:5">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="D13" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:5">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E14" s="3" t="s">
+      <c r="D14" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:5">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E15" s="2" t="s">
+      <c r="D15" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:5">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E16" s="3" t="s">
+      <c r="D16" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:5">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E17" s="2" t="s">
+      <c r="D17" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:5">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E18" s="3" t="s">
+      <c r="D18" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:5">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E19" s="2" t="s">
+      <c r="D19" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:5">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E20" s="3" t="s">
+      <c r="D20" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" s="4" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:5">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E21" s="2" t="s">
+      <c r="D21" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:5">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E22" s="3" t="s">
+      <c r="D22" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" s="4" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E23" s="2" t="s">
+      <c r="D23" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E23" s="3" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:5">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E24" s="3" t="s">
+      <c r="D24" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E25" s="2" t="s">
+      <c r="D25" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:5">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E26" s="3" t="s">
+      <c r="D26" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E26" s="4" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:5">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E27" s="2" t="s">
+      <c r="D27" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:5">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E28" s="3" t="s">
+      <c r="D28" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E29" s="2" t="s">
+      <c r="D29" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1" spans="1:5">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D30" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E30" s="3" t="s">
+      <c r="D30" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1" spans="1:5">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E31" s="2" t="s">
+      <c r="D31" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E31" s="3" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" spans="1:5">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="D32" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E32" s="3" t="s">
+      <c r="D32" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>284</v>
       </c>
     </row>
@@ -4482,7 +4493,7 @@
       <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>295</v>
       </c>
       <c r="C2" t="s">
@@ -4493,7 +4504,7 @@
       <c r="A3" t="s">
         <v>68</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>297</v>
       </c>
       <c r="C3" t="s">
@@ -4504,7 +4515,7 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>298</v>
       </c>
       <c r="C4" t="s">
@@ -4515,7 +4526,7 @@
       <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>299</v>
       </c>
       <c r="C5" t="s">
@@ -4526,7 +4537,7 @@
       <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>300</v>
       </c>
       <c r="C6" t="s">
@@ -4537,7 +4548,7 @@
       <c r="A7" t="s">
         <v>20</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>300</v>
       </c>
       <c r="C7" t="s">
@@ -4548,19 +4559,19 @@
       <c r="A8" t="s">
         <v>50</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>301</v>
       </c>
       <c r="C8" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" ht="28.8" spans="1:3">
       <c r="A9" t="s">
         <v>59</v>
       </c>
-      <c r="B9" t="s">
-        <v>298</v>
+      <c r="B9" s="2" t="s">
+        <v>302</v>
       </c>
       <c r="C9" t="s">
         <v>296</v>
@@ -4570,8 +4581,8 @@
       <c r="A10" t="s">
         <v>24</v>
       </c>
-      <c r="B10" t="s">
-        <v>302</v>
+      <c r="B10" s="2" t="s">
+        <v>303</v>
       </c>
       <c r="C10" t="s">
         <v>296</v>
@@ -4581,8 +4592,8 @@
       <c r="A11" t="s">
         <v>33</v>
       </c>
-      <c r="B11" t="s">
-        <v>303</v>
+      <c r="B11" s="2" t="s">
+        <v>304</v>
       </c>
       <c r="C11" t="s">
         <v>296</v>
@@ -4592,8 +4603,8 @@
       <c r="A12" t="s">
         <v>47</v>
       </c>
-      <c r="B12" t="s">
-        <v>304</v>
+      <c r="B12" s="2" t="s">
+        <v>305</v>
       </c>
       <c r="C12" t="s">
         <v>296</v>
@@ -4603,8 +4614,8 @@
       <c r="A13" t="s">
         <v>40</v>
       </c>
-      <c r="B13" t="s">
-        <v>305</v>
+      <c r="B13" s="2" t="s">
+        <v>306</v>
       </c>
       <c r="C13" t="s">
         <v>296</v>
@@ -4614,8 +4625,8 @@
       <c r="A14" t="s">
         <v>44</v>
       </c>
-      <c r="B14" t="s">
-        <v>306</v>
+      <c r="B14" s="2" t="s">
+        <v>307</v>
       </c>
       <c r="C14" t="s">
         <v>296</v>
@@ -4625,66 +4636,66 @@
       <c r="A15" t="s">
         <v>27</v>
       </c>
-      <c r="B15" t="s">
-        <v>307</v>
+      <c r="B15" s="2" t="s">
+        <v>308</v>
       </c>
       <c r="C15" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>37</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="C16" t="s">
         <v>309</v>
-      </c>
-      <c r="C16" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>310</v>
-      </c>
-      <c r="B17" t="s">
         <v>311</v>
       </c>
+      <c r="B17" s="2" t="s">
+        <v>312</v>
+      </c>
       <c r="C17" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>314</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C18" t="s">
         <v>313</v>
-      </c>
-      <c r="B18" t="s">
-        <v>314</v>
-      </c>
-      <c r="C18" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>62</v>
       </c>
-      <c r="B19" t="s">
-        <v>315</v>
+      <c r="B19" s="2" t="s">
+        <v>316</v>
       </c>
       <c r="C19" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>65</v>
       </c>
-      <c r="B20" t="s">
-        <v>316</v>
+      <c r="B20" s="2" t="s">
+        <v>317</v>
       </c>
       <c r="C20" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemented the Details grid data issues.
</commit_message>
<xml_diff>
--- a/python/table_metadata.xlsx
+++ b/python/table_metadata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9840" activeTab="3"/>
+    <workbookView windowWidth="23040" windowHeight="9840" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -512,7 +512,7 @@
     <t>IsActive</t>
   </si>
   <si>
-    <t>Boolean — TRUE means user is active/enabled. USE = true TO FILTER ACTIVE USERS.</t>
+    <t>Boolean — TRUE means user is active. ALWAYS filter with BOTH: "AbpUsers"."IsActive" = true AND "AbpUsers"."IsDeleted" = false together — never use IsActive alone.</t>
   </si>
   <si>
     <t>Soft delete boolean. Use = false for non-deleted users.</t>
@@ -758,7 +758,7 @@
     <t>Soft delete. Always write "WorkOrders"."IsDeleted" = false — never bare "IsDeleted".</t>
   </si>
   <si>
-    <t>Soft delete. Always write "AbpUsers"."IsDeleted" = false — never bare "IsDeleted"</t>
+    <t>Soft delete. ALWAYS combine with IsActive: use "AbpUsers"."IsActive" = true AND "AbpUsers"."IsDeleted" = false together in every query involving users.</t>
   </si>
   <si>
     <t>Soft delete. Always write "AbpOrganizationUnits"."IsDeleted" = false — never bare "IsDeleted"</t>
@@ -2353,7 +2353,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1" spans="1:4">
+    <row r="2" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1" spans="1:4">
+    <row r="3" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -2381,7 +2381,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1" spans="1:4">
+    <row r="4" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" spans="1:4">
+    <row r="5" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" spans="1:4">
+    <row r="6" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="D6" s="4"/>
     </row>
-    <row r="7" ht="30" customHeight="1" spans="1:4">
+    <row r="7" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
@@ -2435,7 +2435,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1" spans="1:4">
+    <row r="8" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A8" s="3" t="s">
         <v>4</v>
       </c>
@@ -2449,7 +2449,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1" spans="1:4">
+    <row r="9" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A9" s="4" t="s">
         <v>4</v>
       </c>
@@ -2463,7 +2463,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1" spans="1:4">
+    <row r="10" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A10" s="3" t="s">
         <v>4</v>
       </c>
@@ -2477,7 +2477,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1" spans="1:4">
+    <row r="11" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
@@ -2491,7 +2491,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1" spans="1:4">
+    <row r="12" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A12" s="4" t="s">
         <v>4</v>
       </c>
@@ -2505,7 +2505,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1" spans="1:4">
+    <row r="13" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A13" s="4" t="s">
         <v>4</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1" spans="1:4">
+    <row r="14" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
@@ -2533,7 +2533,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" spans="1:4">
+    <row r="15" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A15" s="3" t="s">
         <v>4</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1" spans="1:4">
+    <row r="16" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -2561,7 +2561,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1" spans="1:4">
+    <row r="17" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A17" s="4" t="s">
         <v>4</v>
       </c>
@@ -2575,7 +2575,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1" spans="1:4">
+    <row r="18" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A18" s="3" t="s">
         <v>4</v>
       </c>
@@ -2589,7 +2589,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1" spans="1:4">
+    <row r="19" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A19" s="4" t="s">
         <v>4</v>
       </c>
@@ -2883,7 +2883,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="40" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="40" ht="30" customHeight="1" spans="1:4">
       <c r="A40" s="3" t="s">
         <v>12</v>
       </c>
@@ -2897,7 +2897,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="41" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="41" ht="30" customHeight="1" spans="1:4">
       <c r="A41" s="4" t="s">
         <v>12</v>
       </c>
@@ -2911,7 +2911,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="42" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="42" ht="30" customHeight="1" spans="1:4">
       <c r="A42" s="3" t="s">
         <v>12</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="43" ht="30" customHeight="1" spans="1:4">
       <c r="A43" s="4" t="s">
         <v>12</v>
       </c>
@@ -2939,7 +2939,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="44" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="44" ht="30" customHeight="1" spans="1:4">
       <c r="A44" s="3" t="s">
         <v>12</v>
       </c>
@@ -2953,7 +2953,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="45" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="45" ht="30" customHeight="1" spans="1:4">
       <c r="A45" s="4" t="s">
         <v>12</v>
       </c>
@@ -2967,7 +2967,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="46" ht="30" customHeight="1" spans="1:4">
       <c r="A46" s="3" t="s">
         <v>12</v>
       </c>
@@ -2981,7 +2981,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="47" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="47" ht="30" customHeight="1" spans="1:4">
       <c r="A47" s="4" t="s">
         <v>12</v>
       </c>
@@ -2995,7 +2995,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="48" ht="30" hidden="1" customHeight="1" spans="1:4">
+    <row r="48" ht="30" customHeight="1" spans="1:4">
       <c r="A48" s="3" t="s">
         <v>12</v>
       </c>
@@ -3303,7 +3303,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="70" ht="30" customHeight="1" spans="1:4">
+    <row r="70" ht="30" hidden="1" customHeight="1" spans="1:4">
       <c r="A70" t="s">
         <v>4</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="73" spans="1:4">
+    <row r="73" hidden="1" spans="1:4">
       <c r="A73" t="s">
         <v>4</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="90" ht="72" spans="1:4">
+    <row r="90" ht="72" hidden="1" spans="1:4">
       <c r="A90" t="s">
         <v>4</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="91" spans="1:4">
+    <row r="91" hidden="1" spans="1:4">
       <c r="A91" t="s">
         <v>4</v>
       </c>
@@ -3685,7 +3685,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="102" spans="1:4">
+    <row r="102" hidden="1" spans="1:4">
       <c r="A102" t="s">
         <v>4</v>
       </c>
@@ -3696,7 +3696,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="103" hidden="1" spans="1:4">
+    <row r="103" ht="28.8" spans="1:4">
       <c r="A103" t="s">
         <v>12</v>
       </c>
@@ -3762,7 +3762,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="109" spans="1:4">
+    <row r="109" hidden="1" spans="1:4">
       <c r="A109" t="s">
         <v>4</v>
       </c>
@@ -3776,9 +3776,9 @@
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D109" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
-      <customFilters>
-        <customFilter operator="equal" val="WorkOrders"/>
-      </customFilters>
+      <filters>
+        <filter val="AbpUsers"/>
+      </filters>
     </filterColumn>
     <extLst/>
   </autoFilter>

</xml_diff>

<commit_message>
Fixed the input search and fixed the default chart visibility issue
</commit_message>
<xml_diff>
--- a/python/table_metadata.xlsx
+++ b/python/table_metadata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9840" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="9840"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Triggers" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Columns!$A$1:$D$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Columns!$A$1:$D$108</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="317">
   <si>
     <t>TableName</t>
   </si>
@@ -89,7 +89,7 @@
     <t>UserName</t>
   </si>
   <si>
-    <t>IsActive=true for active users. Use UserName for filtering by login. Name+Surname for full name. To get users by role JOIN AbpUserRoles then AbpRoles.</t>
+    <t>ALWAYS filter users with BOTH conditions together: "AbpUsers"."IsActive" = true AND "AbpUsers"."IsDeleted" = false — never use IsActive alone without IsDeleted. Use UserName for filtering by login. Name+Surname for full name. To get users by role JOIN AbpUserRoles then AbpRoles.</t>
   </si>
   <si>
     <t>AbpRoles</t>
@@ -513,9 +513,6 @@
   </si>
   <si>
     <t>Boolean — TRUE means user is active. ALWAYS filter with BOTH: "AbpUsers"."IsActive" = true AND "AbpUsers"."IsDeleted" = false together — never use IsActive alone.</t>
-  </si>
-  <si>
-    <t>Soft delete boolean. Use = false for non-deleted users.</t>
   </si>
   <si>
     <t>DefaultRole</t>
@@ -2330,7 +2327,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:D109"/>
+  <dimension ref="A1:D108"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2968,388 +2965,385 @@
       </c>
     </row>
     <row r="46" ht="30" customHeight="1" spans="1:4">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1" spans="1:4">
+      <c r="A47" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="48" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A48" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="49" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A49" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="50" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A50" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="51" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A51" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B51" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C46" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="47" ht="30" customHeight="1" spans="1:4">
-      <c r="A47" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="C47" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1" spans="1:4">
-      <c r="A48" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="49" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A49" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="50" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A50" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B50" s="3" t="s">
+      <c r="C51" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="52" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A52" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="53" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A53" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="54" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A54" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="55" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A55" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="56" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A56" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="57" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A57" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="58" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A58" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="59" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A59" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="60" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A60" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="61" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A61" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="62" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A62" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="63" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A63" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="64" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A64" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="65" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A65" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="66" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A66" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="67" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A67" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="68" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A68" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="69" ht="30" hidden="1" customHeight="1" spans="1:4">
+      <c r="A69" t="s">
+        <v>4</v>
+      </c>
+      <c r="B69" t="s">
+        <v>121</v>
+      </c>
+      <c r="C69" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="70" ht="28.8" hidden="1" spans="1:4">
+      <c r="A70" t="s">
+        <v>59</v>
+      </c>
+      <c r="B70" t="s">
         <v>18</v>
       </c>
-      <c r="C50" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="51" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A51" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="52" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A52" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="53" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A53" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="54" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A54" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="55" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A55" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="56" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A56" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="57" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A57" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="D57" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="58" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A58" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="59" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A59" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C59" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="60" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A60" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="61" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A61" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="D61" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="62" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A62" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="63" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A63" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C63" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="64" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A64" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="65" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A65" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="C65" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="D65" s="4" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="66" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A66" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="67" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A67" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B67" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C67" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="D67" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="68" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A68" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="69" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A69" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B69" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C69" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="70" ht="30" hidden="1" customHeight="1" spans="1:4">
-      <c r="A70" t="s">
-        <v>4</v>
-      </c>
-      <c r="B70" t="s">
-        <v>121</v>
-      </c>
-      <c r="C70" s="8" t="s">
+      <c r="C70" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="D70" s="12" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="71" ht="28.8" hidden="1" spans="1:4">
+    </row>
+    <row r="71" hidden="1" spans="1:4">
       <c r="A71" t="s">
         <v>59</v>
       </c>
       <c r="B71" t="s">
-        <v>18</v>
-      </c>
-      <c r="C71" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="C71" s="5" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="72" hidden="1" spans="1:4">
       <c r="A72" t="s">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="B72" t="s">
-        <v>136</v>
-      </c>
-      <c r="C72" s="5" t="s">
         <v>196</v>
+      </c>
+      <c r="C72" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="D72" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="73" hidden="1" spans="1:4">
       <c r="A73" t="s">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="B73" t="s">
-        <v>197</v>
-      </c>
-      <c r="C73" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="D73" t="s">
+        <v>74</v>
+      </c>
+      <c r="C73" s="5" t="s">
         <v>199</v>
       </c>
     </row>
@@ -3358,9 +3352,9 @@
         <v>50</v>
       </c>
       <c r="B74" t="s">
-        <v>74</v>
-      </c>
-      <c r="C74" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C74" s="10" t="s">
         <v>200</v>
       </c>
     </row>
@@ -3369,18 +3363,18 @@
         <v>50</v>
       </c>
       <c r="B75" t="s">
-        <v>52</v>
-      </c>
-      <c r="C75" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C75" s="5" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="76" hidden="1" spans="1:4">
       <c r="A76" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="B76" t="s">
-        <v>129</v>
+        <v>74</v>
       </c>
       <c r="C76" s="5" t="s">
         <v>202</v>
@@ -3391,9 +3385,9 @@
         <v>59</v>
       </c>
       <c r="B77" t="s">
-        <v>74</v>
-      </c>
-      <c r="C77" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C77" s="10" t="s">
         <v>203</v>
       </c>
     </row>
@@ -3402,10 +3396,13 @@
         <v>59</v>
       </c>
       <c r="B78" t="s">
-        <v>18</v>
-      </c>
-      <c r="C78" s="10" t="s">
         <v>204</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="D78" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="79" hidden="1" spans="1:4">
@@ -3413,13 +3410,10 @@
         <v>59</v>
       </c>
       <c r="B79" t="s">
-        <v>205</v>
+        <v>136</v>
       </c>
       <c r="C79" s="5" t="s">
         <v>206</v>
-      </c>
-      <c r="D79" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="80" hidden="1" spans="1:4">
@@ -3427,7 +3421,7 @@
         <v>59</v>
       </c>
       <c r="B80" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C80" s="5" t="s">
         <v>207</v>
@@ -3435,13 +3429,16 @@
     </row>
     <row r="81" hidden="1" spans="1:4">
       <c r="A81" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B81" t="s">
-        <v>129</v>
+        <v>168</v>
       </c>
       <c r="C81" s="5" t="s">
         <v>208</v>
+      </c>
+      <c r="D81" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="82" hidden="1" spans="1:4">
@@ -3449,13 +3446,13 @@
         <v>62</v>
       </c>
       <c r="B82" t="s">
-        <v>169</v>
+        <v>209</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D82" t="s">
-        <v>171</v>
+        <v>123</v>
       </c>
     </row>
     <row r="83" hidden="1" spans="1:4">
@@ -3463,24 +3460,21 @@
         <v>62</v>
       </c>
       <c r="B83" t="s">
-        <v>210</v>
+        <v>129</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="D83" t="s">
-        <v>123</v>
+        <v>185</v>
       </c>
     </row>
     <row r="84" hidden="1" spans="1:4">
       <c r="A84" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B84" t="s">
-        <v>129</v>
+        <v>74</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>186</v>
+        <v>165</v>
       </c>
     </row>
     <row r="85" hidden="1" spans="1:4">
@@ -3488,10 +3482,10 @@
         <v>65</v>
       </c>
       <c r="B85" t="s">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>166</v>
+        <v>211</v>
       </c>
     </row>
     <row r="86" hidden="1" spans="1:4">
@@ -3499,10 +3493,10 @@
         <v>65</v>
       </c>
       <c r="B86" t="s">
-        <v>42</v>
+        <v>212</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="87" hidden="1" spans="1:4">
@@ -3510,10 +3504,13 @@
         <v>65</v>
       </c>
       <c r="B87" t="s">
-        <v>213</v>
+        <v>168</v>
       </c>
       <c r="C87" s="5" t="s">
         <v>214</v>
+      </c>
+      <c r="D87" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="88" hidden="1" spans="1:4">
@@ -3521,49 +3518,46 @@
         <v>65</v>
       </c>
       <c r="B88" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C88" s="5" t="s">
         <v>215</v>
       </c>
       <c r="D88" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="89" hidden="1" spans="1:4">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="89" ht="72" hidden="1" spans="1:4">
       <c r="A89" t="s">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="B89" t="s">
-        <v>167</v>
-      </c>
-      <c r="C89" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D89" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="90" ht="72" hidden="1" spans="1:4">
+      <c r="C89" s="10" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="90" hidden="1" spans="1:4">
       <c r="A90" t="s">
         <v>4</v>
       </c>
       <c r="B90" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C90" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="91" hidden="1" spans="1:4">
       <c r="A91" t="s">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="B91" t="s">
-        <v>219</v>
-      </c>
-      <c r="C91" s="10" t="s">
         <v>220</v>
+      </c>
+      <c r="C91" s="5" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="92" hidden="1" spans="1:4">
@@ -3571,10 +3565,10 @@
         <v>68</v>
       </c>
       <c r="B92" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="93" hidden="1" spans="1:4">
@@ -3582,10 +3576,10 @@
         <v>68</v>
       </c>
       <c r="B93" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="94" hidden="1" spans="1:4">
@@ -3593,10 +3587,10 @@
         <v>68</v>
       </c>
       <c r="B94" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="95" hidden="1" spans="1:4">
@@ -3604,7 +3598,7 @@
         <v>68</v>
       </c>
       <c r="B95" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="C95" s="5" t="s">
         <v>228</v>
@@ -3615,10 +3609,10 @@
         <v>68</v>
       </c>
       <c r="B96" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="97" hidden="1" spans="1:4">
@@ -3626,24 +3620,27 @@
         <v>68</v>
       </c>
       <c r="B97" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="98" hidden="1" spans="1:4">
+        <v>232</v>
+      </c>
+      <c r="D97" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="98" ht="28.8" hidden="1" spans="1:4">
       <c r="A98" t="s">
         <v>68</v>
       </c>
       <c r="B98" t="s">
-        <v>232</v>
-      </c>
-      <c r="C98" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C98" s="10" t="s">
         <v>233</v>
       </c>
       <c r="D98" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
     </row>
     <row r="99" ht="28.8" hidden="1" spans="1:4">
@@ -3651,7 +3648,7 @@
         <v>68</v>
       </c>
       <c r="B99" t="s">
-        <v>124</v>
+        <v>87</v>
       </c>
       <c r="C99" s="10" t="s">
         <v>234</v>
@@ -3660,23 +3657,20 @@
         <v>89</v>
       </c>
     </row>
-    <row r="100" ht="28.8" hidden="1" spans="1:4">
+    <row r="100" hidden="1" spans="1:4">
       <c r="A100" t="s">
         <v>68</v>
       </c>
       <c r="B100" t="s">
-        <v>87</v>
+        <v>129</v>
       </c>
       <c r="C100" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="D100" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="101" hidden="1" spans="1:4">
       <c r="A101" t="s">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="B101" t="s">
         <v>129</v>
@@ -3685,9 +3679,9 @@
         <v>236</v>
       </c>
     </row>
-    <row r="102" hidden="1" spans="1:4">
+    <row r="102" ht="28.8" spans="1:4">
       <c r="A102" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B102" t="s">
         <v>129</v>
@@ -3696,9 +3690,9 @@
         <v>237</v>
       </c>
     </row>
-    <row r="103" ht="28.8" spans="1:4">
+    <row r="103" hidden="1" spans="1:4">
       <c r="A103" t="s">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="B103" t="s">
         <v>129</v>
@@ -3709,7 +3703,7 @@
     </row>
     <row r="104" hidden="1" spans="1:4">
       <c r="A104" t="s">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="B104" t="s">
         <v>129</v>
@@ -3720,7 +3714,7 @@
     </row>
     <row r="105" hidden="1" spans="1:4">
       <c r="A105" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="B105" t="s">
         <v>129</v>
@@ -3731,7 +3725,7 @@
     </row>
     <row r="106" hidden="1" spans="1:4">
       <c r="A106" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B106" t="s">
         <v>129</v>
@@ -3742,7 +3736,7 @@
     </row>
     <row r="107" hidden="1" spans="1:4">
       <c r="A107" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B107" t="s">
         <v>129</v>
@@ -3753,28 +3747,17 @@
     </row>
     <row r="108" hidden="1" spans="1:4">
       <c r="A108" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="B108" t="s">
-        <v>129</v>
-      </c>
-      <c r="C108" s="10" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="109" hidden="1" spans="1:4">
-      <c r="A109" t="s">
-        <v>4</v>
-      </c>
-      <c r="B109" t="s">
+      <c r="C108" t="s">
         <v>244</v>
       </c>
-      <c r="C109" t="s">
-        <v>245</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D109" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D108" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
       <filters>
         <filter val="AbpUsers"/>
@@ -3800,19 +3783,19 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:5">
       <c r="A1" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:5">
@@ -3829,7 +3812,7 @@
         <v>74</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:5">
@@ -3846,7 +3829,7 @@
         <v>74</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:5">
@@ -3863,7 +3846,7 @@
         <v>74</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:5">
@@ -3880,7 +3863,7 @@
         <v>74</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:5">
@@ -3897,7 +3880,7 @@
         <v>74</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:5">
@@ -3914,7 +3897,7 @@
         <v>74</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:5">
@@ -3922,7 +3905,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>50</v>
@@ -3931,7 +3914,7 @@
         <v>74</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:5">
@@ -3939,16 +3922,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:5">
@@ -3959,13 +3942,13 @@
         <v>94</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>261</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:5">
@@ -3976,13 +3959,13 @@
         <v>97</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>263</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:5">
@@ -3999,7 +3982,7 @@
         <v>74</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:5">
@@ -4016,7 +3999,7 @@
         <v>74</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:5">
@@ -4033,7 +4016,7 @@
         <v>74</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:5">
@@ -4050,7 +4033,7 @@
         <v>74</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:5">
@@ -4067,7 +4050,7 @@
         <v>74</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:5">
@@ -4075,7 +4058,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>12</v>
@@ -4084,7 +4067,7 @@
         <v>74</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:5">
@@ -4092,7 +4075,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>16</v>
@@ -4101,7 +4084,7 @@
         <v>74</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:5">
@@ -4109,7 +4092,7 @@
         <v>24</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>4</v>
@@ -4118,7 +4101,7 @@
         <v>74</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:5">
@@ -4126,7 +4109,7 @@
         <v>24</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>47</v>
@@ -4135,7 +4118,7 @@
         <v>74</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:5">
@@ -4143,7 +4126,7 @@
         <v>24</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>33</v>
@@ -4152,7 +4135,7 @@
         <v>74</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:5">
@@ -4160,7 +4143,7 @@
         <v>24</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>12</v>
@@ -4169,7 +4152,7 @@
         <v>74</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5">
@@ -4177,7 +4160,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>4</v>
@@ -4186,7 +4169,7 @@
         <v>74</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:5">
@@ -4194,7 +4177,7 @@
         <v>27</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>12</v>
@@ -4203,7 +4186,7 @@
         <v>74</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5">
@@ -4211,7 +4194,7 @@
         <v>30</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>4</v>
@@ -4220,7 +4203,7 @@
         <v>74</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:5">
@@ -4228,7 +4211,7 @@
         <v>30</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>44</v>
@@ -4237,7 +4220,7 @@
         <v>74</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:5">
@@ -4245,16 +4228,16 @@
         <v>33</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C27" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>278</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:5">
@@ -4271,7 +4254,7 @@
         <v>74</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5">
@@ -4279,7 +4262,7 @@
         <v>37</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>4</v>
@@ -4288,7 +4271,7 @@
         <v>74</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1" spans="1:5">
@@ -4296,7 +4279,7 @@
         <v>37</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>47</v>
@@ -4305,7 +4288,7 @@
         <v>74</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1" spans="1:5">
@@ -4313,7 +4296,7 @@
         <v>37</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>12</v>
@@ -4322,7 +4305,7 @@
         <v>74</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" spans="1:5">
@@ -4333,13 +4316,13 @@
         <v>144</v>
       </c>
       <c r="C32" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>283</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -4356,7 +4339,7 @@
         <v>74</v>
       </c>
       <c r="E33" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -4364,16 +4347,16 @@
         <v>4</v>
       </c>
       <c r="B34" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C34" t="s">
+        <v>285</v>
+      </c>
+      <c r="D34" t="s">
+        <v>74</v>
+      </c>
+      <c r="E34" t="s">
         <v>286</v>
-      </c>
-      <c r="D34" t="s">
-        <v>74</v>
-      </c>
-      <c r="E34" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -4381,7 +4364,7 @@
         <v>62</v>
       </c>
       <c r="B35" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C35" t="s">
         <v>16</v>
@@ -4390,7 +4373,7 @@
         <v>74</v>
       </c>
       <c r="E35" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -4398,7 +4381,7 @@
         <v>62</v>
       </c>
       <c r="B36" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C36" t="s">
         <v>59</v>
@@ -4407,7 +4390,7 @@
         <v>74</v>
       </c>
       <c r="E36" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -4415,7 +4398,7 @@
         <v>65</v>
       </c>
       <c r="B37" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C37" t="s">
         <v>16</v>
@@ -4424,7 +4407,7 @@
         <v>74</v>
       </c>
       <c r="E37" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -4432,7 +4415,7 @@
         <v>65</v>
       </c>
       <c r="B38" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C38" t="s">
         <v>12</v>
@@ -4441,7 +4424,7 @@
         <v>74</v>
       </c>
       <c r="E38" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -4449,7 +4432,7 @@
         <v>68</v>
       </c>
       <c r="B39" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C39" t="s">
         <v>68</v>
@@ -4458,7 +4441,7 @@
         <v>74</v>
       </c>
       <c r="E39" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -4483,10 +4466,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>293</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -4494,10 +4477,10 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="C2" t="s">
         <v>295</v>
-      </c>
-      <c r="C2" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -4505,10 +4488,10 @@
         <v>68</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -4516,10 +4499,10 @@
         <v>8</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -4527,10 +4510,10 @@
         <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -4538,10 +4521,10 @@
         <v>16</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -4549,10 +4532,10 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C7" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -4560,10 +4543,10 @@
         <v>50</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C8" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9" ht="28.8" spans="1:3">
@@ -4571,10 +4554,10 @@
         <v>59</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C9" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -4582,10 +4565,10 @@
         <v>24</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -4593,10 +4576,10 @@
         <v>33</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -4604,10 +4587,10 @@
         <v>47</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C12" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -4615,10 +4598,10 @@
         <v>40</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C13" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -4626,10 +4609,10 @@
         <v>44</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -4637,10 +4620,10 @@
         <v>27</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C15" t="s">
         <v>308</v>
-      </c>
-      <c r="C15" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -4648,32 +4631,32 @@
         <v>37</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C16" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
+        <v>310</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" t="s">
         <v>312</v>
-      </c>
-      <c r="C17" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>313</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>315</v>
-      </c>
       <c r="C18" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -4681,10 +4664,10 @@
         <v>62</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C19" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -4692,10 +4675,10 @@
         <v>65</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C20" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>